<commit_message>
Recargas: automotor por VTV y patentamientos, fuentes de cada rubro sin mes fijo
- Automotor ya no usa el perfil de ventas del MRP: VTV por terminación de patente (febrero a noviembre)
  para la flota obligada y aniversario de compra (patentamientos ACARA 2025) para los exentos (6,5 %).
- Edificios, hoteles, industrias, salud y supermercados: fuente de cada uno (CABA Leyes 941, 4631 y
  6116; PBA Ley 14.701, Decretos 4992/90 y 12/2005; Res. SRT 463/09 y 529/09). Ninguna fija un mes: parejo.
- Datos de la estacionalidad en celdas propias (escuelas estatales, patentamientos, flota, % exento).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Recargas.xlsx
+++ b/salida/Recargas.xlsx
@@ -1336,11 +1336,11 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">Cálculo!F30</f>
-        <v>1073.44515880377</v>
+        <v>1119.01482761851</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">Cálculo!I30</f>
-        <v>575.8235761071</v>
+        <v>599.546838706733</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>21</v>
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Cálculo!G30</f>
-        <v>583.719434863009</v>
+        <v>585.256044364544</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">Cálculo!J30</f>
-        <v>321.26184967668</v>
+        <v>322.091098622045</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>21</v>
@@ -1368,11 +1368,11 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1828</v>
+        <v>1833</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>1001</v>
+        <v>1004</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>24</v>
@@ -1384,11 +1384,11 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">Cálculo!E44</f>
-        <v>107.121978748165</v>
+        <v>110.767552253345</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">Cálculo!I44</f>
-        <v>57.883289303567</v>
+        <v>59.7811503115376</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>26</v>
@@ -1400,11 +1400,11 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">Cálculo!B61</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">Cálculo!C61</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>28</v>
@@ -1432,11 +1432,11 @@
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">Cálculo!B64</f>
-        <v>0.923984721900265</v>
+        <v>0.956474196159033</v>
       </c>
       <c r="C13" s="10" t="n">
         <f aca="false">Cálculo!C64</f>
-        <v>0.896545923711903</v>
+        <v>0.93657890101826</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>28</v>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Cálculo!E74</f>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Cálculo!I74</f>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">Cálculo!E75</f>
-        <v>156</v>
+        <v>160.8</v>
       </c>
       <c r="C15" s="11" t="n">
         <f aca="false">Cálculo!I75</f>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Cálculo!E77</f>
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">Cálculo!I77</f>
@@ -1907,52 +1907,52 @@
         <v>109</v>
       </c>
       <c r="B5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E51:P68"")"),0.119933202334914)</f>
-        <v>0.119933202334914</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E55:P72"")"),0.00749080356204596)</f>
+        <v>0.00749080356204596</v>
       </c>
       <c r="C5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0899878549699844)</f>
-        <v>0.0899878549699844</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0980789973414249)</f>
+        <v>0.0980789973414249</v>
       </c>
       <c r="D5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800060725150078)</f>
-        <v>0.0800060725150078</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0986610060682725)</f>
+        <v>0.0986610060682725</v>
       </c>
       <c r="E5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993660972474985)</f>
+        <v>0.0993660972474985</v>
       </c>
       <c r="F5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0700242900600312)</f>
-        <v>0.0700242900600312</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994029049644587)</f>
+        <v>0.0994029049644587</v>
       </c>
       <c r="G5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0700242900600312)</f>
-        <v>0.0700242900600312</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990676994264772)</f>
+        <v>0.0990676994264772</v>
       </c>
       <c r="H5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100122038394086)</f>
+        <v>0.100122038394086</v>
       </c>
       <c r="I5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993285448657443)</f>
+        <v>0.0993285448657443</v>
       </c>
       <c r="J5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994522656022319)</f>
+        <v>0.0994522656022319</v>
       </c>
       <c r="K5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990432318689603)</f>
+        <v>0.0990432318689603</v>
       </c>
       <c r="L5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750151812875195)</f>
-        <v>0.0750151812875195</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0972817804891135)</f>
+        <v>0.0972817804891135</v>
       </c>
       <c r="M5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119933202334914)</f>
-        <v>0.119933202334914</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0027046301696863)</f>
+        <v>0.0027046301696863</v>
       </c>
       <c r="N5" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""datos_base!K2:K18"")"),108842.626397553)</f>
@@ -2101,52 +2101,52 @@
         <v>111</v>
       </c>
       <c r="B7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0828991382713857)</f>
-        <v>0.0828991382713857</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0752806934699069)</f>
+        <v>0.0752806934699069</v>
       </c>
       <c r="C7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.115838094188612)</f>
-        <v>0.115838094188612</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.116386303068985)</f>
+        <v>0.116386303068985</v>
       </c>
       <c r="D7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.080193907522717)</f>
-        <v>0.080193907522717</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0814578576260751)</f>
+        <v>0.0814578576260751</v>
       </c>
       <c r="E7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815056305150171)</f>
+        <v>0.0815056305150171</v>
       </c>
       <c r="F7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795175998355498)</f>
-        <v>0.0795175998355498</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815081243924422)</f>
+        <v>0.0815081243924422</v>
       </c>
       <c r="G7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795175998355498)</f>
-        <v>0.0795175998355498</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0814854128093016)</f>
+        <v>0.0814854128093016</v>
       </c>
       <c r="H7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815568487028296)</f>
+        <v>0.0815568487028296</v>
       </c>
       <c r="I7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815030861834244)</f>
+        <v>0.0815030861834244</v>
       </c>
       <c r="J7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815114687829777)</f>
+        <v>0.0815114687829777</v>
       </c>
       <c r="K7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0814837550295103)</f>
+        <v>0.0814837550295103</v>
       </c>
       <c r="L7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798557536791334)</f>
-        <v>0.0798557536791334</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0813644093000141)</f>
+        <v>0.0813644093000141</v>
       </c>
       <c r="M7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0828991382713857)</f>
-        <v>0.0828991382713857</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0749564101195165)</f>
+        <v>0.0749564101195165</v>
       </c>
       <c r="N7" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),56059.2707104735)</f>
@@ -2157,8 +2157,8 @@
         <v>1</v>
       </c>
       <c r="P7" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1010)</f>
-        <v>1010</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1015)</f>
+        <v>1015</v>
       </c>
       <c r="Q7" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),69628)</f>
@@ -3556,52 +3556,52 @@
         <v>126</v>
       </c>
       <c r="B22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101766211787366)</f>
-        <v>0.101766211787366</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0403512821171889)</f>
+        <v>0.0403512821171889</v>
       </c>
       <c r="C22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.104101668275449)</f>
-        <v>0.104101668275449</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108520970470319)</f>
+        <v>0.108520970470319</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0799584071106368)</f>
-        <v>0.0799584071106368</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0901475479034248)</f>
+        <v>0.0901475479034248</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905326617542125)</f>
+        <v>0.0905326617542125</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0745064559414546)</f>
-        <v>0.0745064559414546</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905527657663388)</f>
+        <v>0.0905527657663388</v>
       </c>
       <c r="G22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0745064559414546)</f>
-        <v>0.0745064559414546</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0903696798061951)</f>
+        <v>0.0903696798061951</v>
       </c>
       <c r="H22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0909455493558567)</f>
+        <v>0.0909455493558567</v>
       </c>
       <c r="I22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905121510135173)</f>
+        <v>0.0905121510135173</v>
       </c>
       <c r="J22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905797260600571)</f>
+        <v>0.0905797260600571</v>
       </c>
       <c r="K22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0903563158674985)</f>
+        <v>0.0903563158674985</v>
       </c>
       <c r="L22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0772324315260457)</f>
-        <v>0.0772324315260457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0893942284895046)</f>
+        <v>0.0893942284895046</v>
       </c>
       <c r="M22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101766211787366)</f>
-        <v>0.101766211787366</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0377371213958866)</f>
+        <v>0.0377371213958866</v>
       </c>
       <c r="N22" s="7" t="n">
         <f aca="false">SUM(N5:N21)</f>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="P22" s="7" t="n">
         <f aca="false">SUM(P5:P21)</f>
-        <v>1828</v>
+        <v>1833</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3709,52 +3709,52 @@
         <v>101</v>
       </c>
       <c r="B28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E35:P41"")"),0.12)</f>
-        <v>0.12</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E35:P41"")"),0.00735238492719494)</f>
+        <v>0.00735238492719494</v>
       </c>
       <c r="C28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.09)</f>
-        <v>0.09</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0981059093482913)</f>
+        <v>0.0981059093482913</v>
       </c>
       <c r="D28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0986889802872471)</f>
+        <v>0.0986889802872471</v>
       </c>
       <c r="E28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993953583138234)</f>
+        <v>0.0993953583138234</v>
       </c>
       <c r="F28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.07)</f>
-        <v>0.07</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994322332077878)</f>
+        <v>0.0994322332077878</v>
       </c>
       <c r="G28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.07)</f>
-        <v>0.07</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990964158931013)</f>
+        <v>0.0990964158931013</v>
       </c>
       <c r="H28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100152679112986)</f>
+        <v>0.100152679112986</v>
       </c>
       <c r="I28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993577373959928)</f>
+        <v>0.0993577373959928</v>
       </c>
       <c r="J28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994816839326416)</f>
+        <v>0.0994816839326416</v>
       </c>
       <c r="K28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990719036803504)</f>
+        <v>0.0990719036803504</v>
       </c>
       <c r="L28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0973072375119662)</f>
+        <v>0.0973072375119662</v>
       </c>
       <c r="M28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.12)</f>
-        <v>0.12</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.00255747638861682)</f>
+        <v>0.00255747638861682</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4159,52 +4159,52 @@
         <v>109</v>
       </c>
       <c r="B39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E51:P68"")"),0.119942566698092)</f>
-        <v>0.119942566698092</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E55:P72"")"),0.00747139865671394)</f>
+        <v>0.00747139865671394</v>
       </c>
       <c r="C39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0899895575814713)</f>
-        <v>0.0899895575814713</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0980827701350671)</f>
+        <v>0.0980827701350671</v>
       </c>
       <c r="D39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800052212092643)</f>
-        <v>0.0800052212092643</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0986649277734065)</f>
+        <v>0.0986649277734065</v>
       </c>
       <c r="E39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993701993557339)</f>
+        <v>0.0993701993557339</v>
       </c>
       <c r="F39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0700208848370573)</f>
-        <v>0.0700208848370573</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994070164902368)</f>
+        <v>0.0994070164902368</v>
       </c>
       <c r="G39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0700208848370573)</f>
-        <v>0.0700208848370573</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990717251872927)</f>
+        <v>0.0990717251872927</v>
       </c>
       <c r="H39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100126333915785)</f>
+        <v>0.100126333915785</v>
       </c>
       <c r="I39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993326373659087)</f>
+        <v>0.0993326373659087</v>
       </c>
       <c r="J39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994563897573158)</f>
+        <v>0.0994563897573158</v>
       </c>
       <c r="K39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990472513695595)</f>
+        <v>0.0990472513695595</v>
       </c>
       <c r="L39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0750130530231608)</f>
-        <v>0.0750130530231608</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0972853493085793)</f>
+        <v>0.0972853493085793</v>
       </c>
       <c r="M39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119942566698092)</f>
-        <v>0.119942566698092</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.00268400068440077)</f>
+        <v>0.00268400068440077</v>
       </c>
       <c r="N39" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""datos_base!K2:K18"")"),56575.8368575054)</f>
@@ -4353,52 +4353,52 @@
         <v>111</v>
       </c>
       <c r="B41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0823827818974594)</f>
-        <v>0.0823827818974594</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0744731592432624)</f>
+        <v>0.0744731592432624</v>
       </c>
       <c r="C41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.122577805221806)</f>
-        <v>0.122577805221806</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.123146966709803)</f>
+        <v>0.123146966709803</v>
       </c>
       <c r="D41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795741569126926)</f>
-        <v>0.0795741569126926</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.080886415337057)</f>
+        <v>0.080886415337057</v>
       </c>
       <c r="E41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809360141114104)</f>
+        <v>0.0809360141114104</v>
       </c>
       <c r="F41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788720006665009)</f>
-        <v>0.0788720006665009</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809386033051228)</f>
+        <v>0.0809386033051228</v>
       </c>
       <c r="G41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788720006665009)</f>
-        <v>0.0788720006665009</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809150236826142)</f>
+        <v>0.0809150236826142</v>
       </c>
       <c r="H41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809891898643607)</f>
+        <v>0.0809891898643607</v>
       </c>
       <c r="I41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809333725351661)</f>
+        <v>0.0809333725351661</v>
       </c>
       <c r="J41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809420755186563)</f>
+        <v>0.0809420755186563</v>
       </c>
       <c r="K41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809133025422851)</f>
+        <v>0.0809133025422851</v>
       </c>
       <c r="L41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792230787895967)</f>
-        <v>0.0792230787895967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0807893954050276)</f>
+        <v>0.0807893954050276</v>
       </c>
       <c r="M41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0823827818974594)</f>
-        <v>0.0823827818974594</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741364817452343)</f>
+        <v>0.0741364817452343</v>
       </c>
       <c r="N41" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),29139.3203107948)</f>
@@ -4409,8 +4409,8 @@
         <v>1</v>
       </c>
       <c r="P41" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),551)</f>
-        <v>551</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),554)</f>
+        <v>554</v>
       </c>
       <c r="Q41" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),36760)</f>
@@ -5808,52 +5808,52 @@
         <v>126</v>
       </c>
       <c r="B56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101494630758993)</f>
-        <v>0.101494630758993</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0399853669657492)</f>
+        <v>0.0399853669657492</v>
       </c>
       <c r="C56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.107432404543694)</f>
-        <v>0.107432404543694</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111858494843661)</f>
+        <v>0.111858494843661</v>
       </c>
       <c r="D56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0796533290133718)</f>
-        <v>0.0796533290133718</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0898581204576652)</f>
+        <v>0.0898581204576652</v>
       </c>
       <c r="E56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0902438258482885)</f>
+        <v>0.0902438258482885</v>
       </c>
       <c r="F56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741930035769664)</f>
-        <v>0.0741930035769664</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0902639607404363)</f>
+        <v>0.0902639607404363</v>
       </c>
       <c r="G56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741930035769664)</f>
-        <v>0.0741930035769664</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0900805935578995)</f>
+        <v>0.0900805935578995</v>
       </c>
       <c r="H56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0906573476506073)</f>
+        <v>0.0906573476506073</v>
       </c>
       <c r="I56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0902232836028314)</f>
+        <v>0.0902232836028314</v>
       </c>
       <c r="J56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0902909624455131)</f>
+        <v>0.0902909624455131</v>
       </c>
       <c r="K56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0900672090920209)</f>
+        <v>0.0900672090920209</v>
       </c>
       <c r="L56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0769231662951691)</f>
-        <v>0.0769231662951691</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0891036439354216)</f>
+        <v>0.0891036439354216</v>
       </c>
       <c r="M56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101494630758993)</f>
-        <v>0.101494630758993</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0373671908599057)</f>
+        <v>0.0373671908599057</v>
       </c>
       <c r="N56" s="7" t="n">
         <f aca="false">SUM(N39:N55)</f>
@@ -5861,7 +5861,7 @@
       </c>
       <c r="P56" s="7" t="n">
         <f aca="false">SUM(P39:P55)</f>
-        <v>1001</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5961,52 +5961,52 @@
         <v>101</v>
       </c>
       <c r="B62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E35:P41"")"),0.12)</f>
-        <v>0.12</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E35:P41"")"),0.00735238492719494)</f>
+        <v>0.00735238492719494</v>
       </c>
       <c r="C62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.09)</f>
-        <v>0.09</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0981059093482913)</f>
+        <v>0.0981059093482913</v>
       </c>
       <c r="D62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0986889802872471)</f>
+        <v>0.0986889802872471</v>
       </c>
       <c r="E62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993953583138234)</f>
+        <v>0.0993953583138234</v>
       </c>
       <c r="F62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.07)</f>
-        <v>0.07</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994322332077878)</f>
+        <v>0.0994322332077878</v>
       </c>
       <c r="G62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.07)</f>
-        <v>0.07</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990964158931013)</f>
+        <v>0.0990964158931013</v>
       </c>
       <c r="H62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100152679112986)</f>
+        <v>0.100152679112986</v>
       </c>
       <c r="I62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993577373959928)</f>
+        <v>0.0993577373959928</v>
       </c>
       <c r="J62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994816839326416)</f>
+        <v>0.0994816839326416</v>
       </c>
       <c r="K62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0990719036803504)</f>
+        <v>0.0990719036803504</v>
       </c>
       <c r="L62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.075)</f>
-        <v>0.075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0973072375119662)</f>
+        <v>0.0973072375119662</v>
       </c>
       <c r="M62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.12)</f>
-        <v>0.12</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.00255747638861682)</f>
+        <v>0.00255747638861682</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6440,11 +6440,11 @@
       </c>
       <c r="B7" s="26" t="n">
         <f aca="false">INDEX(Importados!$B$22:$M$22,B5)</f>
-        <v>0.104101668275449</v>
+        <v>0.108520970470319</v>
       </c>
       <c r="C7" s="26" t="n">
         <f aca="false">INDEX(Importados!$B$56:$M$56,C5)</f>
-        <v>0.107432404543694</v>
+        <v>0.111858494843661</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="F13" s="29" t="n">
         <f aca="false">Importados!$N$5*INDEX(Importados!$B$5:$M$5,$B$5)/$B$8</f>
-        <v>489.72572394076</v>
+        <v>533.758783253965</v>
       </c>
       <c r="G13" s="29" t="n">
         <f aca="false">F13*Importados!$O$5</f>
@@ -6593,11 +6593,11 @@
       </c>
       <c r="H13" s="23" t="n">
         <f aca="false">F13/$C13</f>
-        <v>6.80174616584389</v>
+        <v>7.41331643408285</v>
       </c>
       <c r="I13" s="29" t="n">
         <f aca="false">Importados!$N$39*INDEX(Importados!$B$39:$M$39,$C$5)/$C$8</f>
-        <v>254.56172643042</v>
+        <v>277.455740084688</v>
       </c>
       <c r="J13" s="29" t="n">
         <f aca="false">I13*Importados!$O$39</f>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="K13" s="23" t="n">
         <f aca="false">I13/$C13</f>
-        <v>3.53557953375584</v>
+        <v>3.85355194562067</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>151</v>
@@ -6673,27 +6673,27 @@
       </c>
       <c r="F15" s="29" t="n">
         <f aca="false">Importados!$N$7*INDEX(Importados!$B$7:$M$7,$B$5)/$B$8</f>
-        <v>324.689954035236</v>
+        <v>326.226563536772</v>
       </c>
       <c r="G15" s="29" t="n">
         <f aca="false">F15*Importados!$O$7</f>
-        <v>324.689954035236</v>
+        <v>326.226563536772</v>
       </c>
       <c r="H15" s="23" t="n">
         <f aca="false">F15/$C15</f>
-        <v>13.5287480848015</v>
+        <v>13.5927734806988</v>
       </c>
       <c r="I15" s="29" t="n">
         <f aca="false">Importados!$N$41*INDEX(Importados!$B$41:$M$41,$C$5)/$C$8</f>
-        <v>178.591696467621</v>
+        <v>179.420945412987</v>
       </c>
       <c r="J15" s="29" t="n">
         <f aca="false">I15*Importados!$O$41</f>
-        <v>178.591696467621</v>
+        <v>179.420945412987</v>
       </c>
       <c r="K15" s="23" t="n">
         <f aca="false">I15/$C15</f>
-        <v>7.44132068615088</v>
+        <v>7.47587272554111</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>151</v>
@@ -7321,27 +7321,27 @@
       </c>
       <c r="F30" s="30" t="n">
         <f aca="false">SUM(F13:F29)</f>
-        <v>1073.44515880377</v>
+        <v>1119.01482761851</v>
       </c>
       <c r="G30" s="30" t="n">
         <f aca="false">SUM(G13:G29)</f>
-        <v>583.719434863009</v>
+        <v>585.256044364544</v>
       </c>
       <c r="H30" s="30" t="n">
         <f aca="false">SUM(H13:H29)</f>
-        <v>37.3025755918414</v>
+        <v>37.9781712559777</v>
       </c>
       <c r="I30" s="30" t="n">
         <f aca="false">SUM(I13:I29)</f>
-        <v>575.8235761071</v>
+        <v>599.546838706733</v>
       </c>
       <c r="J30" s="30" t="n">
         <f aca="false">SUM(J13:J29)</f>
-        <v>321.26184967668</v>
+        <v>322.091098622045</v>
       </c>
       <c r="K30" s="30" t="n">
         <f aca="false">SUM(K13:K29)</f>
-        <v>20.2315375836849</v>
+        <v>20.58406203494</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7350,11 +7350,11 @@
       </c>
       <c r="F31" s="11" t="n">
         <f aca="false">SUMPRODUCT(F13:F29,$B$13:$B$29)/F30</f>
-        <v>6.85140037194582</v>
+        <v>6.65882736300077</v>
       </c>
       <c r="I31" s="11" t="n">
         <f aca="false">SUMPRODUCT(I13:I29,$B$13:$B$29)/I30</f>
-        <v>6.94428580605528</v>
+        <v>6.75381882934406</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="C37" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$28:$M$28,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$Q$5:$Q$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>505.960530411216</v>
+        <v>551.530199225957</v>
       </c>
       <c r="D37" s="22" t="n">
         <f aca="false">Importados!Q$23</f>
@@ -7437,15 +7437,15 @@
       </c>
       <c r="E37" s="28" t="n">
         <f aca="false">2*C37/D37</f>
-        <v>40.4768424328973</v>
+        <v>44.1224159380766</v>
       </c>
       <c r="F37" s="28" t="n">
         <f aca="false">E37*(Supuestos!$B$16+Supuestos!$B$17)/60+2*C37*$B37/60</f>
-        <v>32.0441669260437</v>
+        <v>34.9302459509773</v>
       </c>
       <c r="G37" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$62:$M$62,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$Q$39:$Q$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>263.399643670702</v>
+        <v>287.122906270335</v>
       </c>
       <c r="H37" s="22" t="n">
         <f aca="false">Importados!Q$57</f>
@@ -7453,11 +7453,11 @@
       </c>
       <c r="I37" s="28" t="n">
         <f aca="false">2*G37/H37</f>
-        <v>21.0719714936561</v>
+        <v>22.9698325016268</v>
       </c>
       <c r="J37" s="28" t="n">
         <f aca="false">I37*(Supuestos!$B$16+Supuestos!$B$17)/60+2*G37*$B37/60</f>
-        <v>16.6819774324778</v>
+        <v>18.1844507304545</v>
       </c>
       <c r="M37" s="5" t="s">
         <v>164</v>
@@ -7727,27 +7727,27 @@
       </c>
       <c r="C44" s="30" t="n">
         <f aca="false">SUM(C37:C43)</f>
-        <v>1073.44515880377</v>
+        <v>1119.01482761851</v>
       </c>
       <c r="E44" s="30" t="n">
         <f aca="false">SUM(E37:E43)</f>
-        <v>107.121978748165</v>
+        <v>110.767552253345</v>
       </c>
       <c r="F44" s="30" t="n">
         <f aca="false">SUM(F37:F43)</f>
-        <v>99.2379374565358</v>
+        <v>102.124016481469</v>
       </c>
       <c r="G44" s="30" t="n">
         <f aca="false">SUM(G37:G43)</f>
-        <v>575.823576107101</v>
+        <v>599.546838706733</v>
       </c>
       <c r="I44" s="30" t="n">
         <f aca="false">SUM(I37:I43)</f>
-        <v>57.883289303567</v>
+        <v>59.7811503115376</v>
       </c>
       <c r="J44" s="30" t="n">
         <f aca="false">SUM(J37:J43)</f>
-        <v>53.7409442783928</v>
+        <v>55.2434175763695</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7784,11 +7784,11 @@
       </c>
       <c r="B49" s="29" t="n">
         <f aca="false">F30</f>
-        <v>1073.44515880377</v>
+        <v>1119.01482761851</v>
       </c>
       <c r="C49" s="29" t="n">
         <f aca="false">I30</f>
-        <v>575.8235761071</v>
+        <v>599.546838706733</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>168</v>
@@ -7809,11 +7809,11 @@
       </c>
       <c r="B50" s="29" t="n">
         <f aca="false">G30</f>
-        <v>583.719434863009</v>
+        <v>585.256044364544</v>
       </c>
       <c r="C50" s="29" t="n">
         <f aca="false">J30</f>
-        <v>321.26184967668</v>
+        <v>322.091098622045</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>168</v>
@@ -7834,11 +7834,11 @@
       </c>
       <c r="B51" s="29" t="n">
         <f aca="false">B49+B50</f>
-        <v>1657.16459366678</v>
+        <v>1704.27087198305</v>
       </c>
       <c r="C51" s="29" t="n">
         <f aca="false">C49+C50</f>
-        <v>897.085425783779</v>
+        <v>921.637937328778</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>170</v>
@@ -7859,11 +7859,11 @@
       </c>
       <c r="B52" s="28" t="n">
         <f aca="false">F31</f>
-        <v>6.85140037194582</v>
+        <v>6.65882736300077</v>
       </c>
       <c r="C52" s="28" t="n">
         <f aca="false">I31</f>
-        <v>6.94428580605528</v>
+        <v>6.75381882934406</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>171</v>
@@ -7884,11 +7884,11 @@
       </c>
       <c r="B53" s="31" t="n">
         <f aca="false">H30/F30</f>
-        <v>0.0347503319437491</v>
+        <v>0.0339389347831994</v>
       </c>
       <c r="C53" s="31" t="n">
         <f aca="false">K30/I30</f>
-        <v>0.035134958732433</v>
+        <v>0.0343327004764821</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>173</v>
@@ -7909,11 +7909,11 @@
       </c>
       <c r="B54" s="21" t="n">
         <f aca="false">Supuestos!$B$6/(B53*Supuestos!$B$22)</f>
-        <v>150.139322778076</v>
+        <v>153.728787826616</v>
       </c>
       <c r="C54" s="21" t="n">
         <f aca="false">Supuestos!$B$6/(C53*Supuestos!$B$22)</f>
-        <v>148.495728828953</v>
+        <v>151.965654665637</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>175</v>
@@ -7934,11 +7934,11 @@
       </c>
       <c r="B55" s="21" t="n">
         <f aca="false">Supuestos!$B$10/B52</f>
-        <v>241.702412660157</v>
+        <v>248.692436329169</v>
       </c>
       <c r="C55" s="21" t="n">
         <f aca="false">Supuestos!$B$10/C52</f>
-        <v>238.4694475789</v>
+        <v>245.194613868674</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>177</v>
@@ -7959,11 +7959,11 @@
       </c>
       <c r="B56" s="21" t="n">
         <f aca="false">MIN(B54,B55)</f>
-        <v>150.139322778076</v>
+        <v>153.728787826616</v>
       </c>
       <c r="C56" s="21" t="n">
         <f aca="false">MIN(C54,C55)</f>
-        <v>148.495728828953</v>
+        <v>151.965654665637</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>179</v>
@@ -7984,11 +7984,11 @@
       </c>
       <c r="B57" s="23" t="n">
         <f aca="false">B51/B56</f>
-        <v>11.0375121121085</v>
+        <v>11.086218112285</v>
       </c>
       <c r="C57" s="23" t="n">
         <f aca="false">C51/C56</f>
-        <v>6.04115305442286</v>
+        <v>6.06477785626375</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>181</v>
@@ -8009,11 +8009,11 @@
       </c>
       <c r="B58" s="28" t="n">
         <f aca="false">E44</f>
-        <v>107.121978748165</v>
+        <v>110.767552253345</v>
       </c>
       <c r="C58" s="28" t="n">
         <f aca="false">I44</f>
-        <v>57.883289303567</v>
+        <v>59.7811503115376</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>182</v>
@@ -8034,11 +8034,11 @@
       </c>
       <c r="B59" s="28" t="n">
         <f aca="false">F44</f>
-        <v>99.2379374565358</v>
+        <v>102.124016481469</v>
       </c>
       <c r="C59" s="28" t="n">
         <f aca="false">J44</f>
-        <v>53.7409442783928</v>
+        <v>55.2434175763695</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>182</v>
@@ -8059,11 +8059,11 @@
       </c>
       <c r="B60" s="23" t="n">
         <f aca="false">B59/($B$9-Supuestos!$B$15)</f>
-        <v>16.539656242756</v>
+        <v>17.0206694135782</v>
       </c>
       <c r="C60" s="23" t="n">
         <f aca="false">C59/($C$9-Supuestos!$B$15)</f>
-        <v>8.95682404639879</v>
+        <v>9.20723626272825</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>185</v>
@@ -8084,11 +8084,11 @@
       </c>
       <c r="B61" s="9" t="n">
         <f aca="false">ROUNDUP(MAX(B57,B60),0)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C61" s="9" t="n">
         <f aca="false">ROUNDUP(MAX(C57,C60),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>186</v>
@@ -8109,11 +8109,11 @@
       </c>
       <c r="B62" s="28" t="n">
         <f aca="false">B61*Supuestos!$B$15+B59</f>
-        <v>124.737937456536</v>
+        <v>129.124016481469</v>
       </c>
       <c r="C62" s="28" t="n">
         <f aca="false">C61*Supuestos!$B$15+C59</f>
-        <v>67.2409442783928</v>
+        <v>70.2434175763695</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>188</v>
@@ -8159,11 +8159,11 @@
       </c>
       <c r="B64" s="32" t="n">
         <f aca="false">B62/(B63*$B$9*Supuestos!$B$14)</f>
-        <v>0.923984721900265</v>
+        <v>0.956474196159033</v>
       </c>
       <c r="C64" s="32" t="n">
         <f aca="false">C62/(C63*$C$9*Supuestos!$B$14)</f>
-        <v>0.896545923711903</v>
+        <v>0.93657890101826</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>191</v>
@@ -8184,11 +8184,11 @@
       </c>
       <c r="B65" s="21" t="n">
         <f aca="false">B51*B52/B61</f>
-        <v>667.876359613176</v>
+        <v>630.469195351441</v>
       </c>
       <c r="C65" s="21" t="n">
         <f aca="false">C51*C52/C61</f>
-        <v>692.17973212104</v>
+        <v>622.457565496893</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>193</v>
@@ -8290,11 +8290,11 @@
       </c>
       <c r="B70" s="21" t="n">
         <f aca="false">F30*Supuestos!$B$20</f>
-        <v>536.722579401884</v>
+        <v>559.507413809255</v>
       </c>
       <c r="C70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*H13:H29)*Supuestos!$B$20*Supuestos!$B$22</f>
-        <v>17.7308598471581</v>
+        <v>18.1193273540365</v>
       </c>
       <c r="D70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*H13:H29)*Supuestos!$B$20</f>
@@ -8302,15 +8302,15 @@
       </c>
       <c r="E70" s="22" t="n">
         <f aca="false">ROUNDUP(C70,0)+ROUNDUP(D70,0)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F70" s="21" t="n">
         <f aca="false">I30*Supuestos!$B$20</f>
-        <v>287.91178805355</v>
+        <v>299.773419353367</v>
       </c>
       <c r="G70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*K13:K29)*Supuestos!$B$20*Supuestos!$B$22</f>
-        <v>9.63985334793126</v>
+        <v>9.84255490740292</v>
       </c>
       <c r="H70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*K13:K29)*Supuestos!$B$20</f>
@@ -8330,11 +8330,11 @@
       </c>
       <c r="B71" s="21" t="n">
         <f aca="false">F30*Supuestos!$B$21</f>
-        <v>536.722579401884</v>
+        <v>559.507413809255</v>
       </c>
       <c r="C71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*H13:H29)*Supuestos!$B$21*Supuestos!$B$22</f>
-        <v>17.7308598471581</v>
+        <v>18.1193273540365</v>
       </c>
       <c r="D71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*H13:H29)*Supuestos!$B$21</f>
@@ -8342,15 +8342,15 @@
       </c>
       <c r="E71" s="22" t="n">
         <f aca="false">ROUNDUP(C71,0)+ROUNDUP(D71,0)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F71" s="21" t="n">
         <f aca="false">I30*Supuestos!$B$21</f>
-        <v>287.91178805355</v>
+        <v>299.773419353367</v>
       </c>
       <c r="G71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*K13:K29)*Supuestos!$B$21*Supuestos!$B$22</f>
-        <v>9.63985334793126</v>
+        <v>9.84255490740292</v>
       </c>
       <c r="H71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*K13:K29)*Supuestos!$B$21</f>
@@ -8370,11 +8370,11 @@
       </c>
       <c r="B72" s="21" t="n">
         <f aca="false">G30</f>
-        <v>583.719434863009</v>
+        <v>585.256044364544</v>
       </c>
       <c r="C72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*G13:G29/$C$13:$C$29)</f>
-        <v>24.0345318292138</v>
+        <v>24.0985572251111</v>
       </c>
       <c r="D72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*G13:G29/$C$13:$C$29)</f>
@@ -8386,11 +8386,11 @@
       </c>
       <c r="F72" s="21" t="n">
         <f aca="false">J30</f>
-        <v>321.26184967668</v>
+        <v>322.091098622045</v>
       </c>
       <c r="G72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*J13:J29/$C$13:$C$29)</f>
-        <v>13.2293828104724</v>
+        <v>13.2639348498627</v>
       </c>
       <c r="H72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*J13:J29/$C$13:$C$29)</f>
@@ -8444,7 +8444,7 @@
       </c>
       <c r="E74" s="9" t="n">
         <f aca="false">SUM(E70:E73)</f>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I74" s="9" t="n">
         <f aca="false">SUM(I70:I73)</f>
@@ -8457,7 +8457,7 @@
       </c>
       <c r="E75" s="11" t="n">
         <f aca="false">E74*Supuestos!$B$26</f>
-        <v>156</v>
+        <v>160.8</v>
       </c>
       <c r="I75" s="11" t="n">
         <f aca="false">I74*Supuestos!$B$26</f>
@@ -8470,11 +8470,11 @@
       </c>
       <c r="E76" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1828</v>
+        <v>1833</v>
       </c>
       <c r="I76" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>1001</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="E77" s="9" t="n">
         <f aca="false">ROUNDUP(SUM(C70:C72),0)+B63*Supuestos!$B$6+E73*Supuestos!$B$25</f>
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I77" s="9" t="n">
         <f aca="false">ROUNDUP(SUM(G70:G72),0)+C63*Supuestos!$B$6+I73*Supuestos!$B$25</f>

</xml_diff>

<commit_message>
Aprovechamientos: ensayo de pérdidas de W-MAN, estatales en 3 meses y puestos de recargas unidos
- Manuales: ensayo de pérdidas en tandas de 6 (40 s, W-MAN); el puesto más cargado pasa a ser la pintura
- Recargas: las escuelas estatales se reparten de febrero a abril (parámetro en B49), en vez de todo en febrero
- Recargas: BC y Clase D con su equipo exclusivo dentro de los puestos de polvo; CO2 y halogenado recuperan y cargan en
  la misma máquina; descarga y carga de líquidos en un solo puesto (23 puestos)
- Corte: regenerado con los sustitutos nuevos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Recargas.xlsx
+++ b/salida/Recargas.xlsx
@@ -1308,11 +1308,11 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1757</v>
+        <v>1384</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>985</v>
+        <v>744</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>23</v>
@@ -1946,16 +1946,16 @@
         <v>0.0789430506992025</v>
       </c>
       <c r="C6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.131626442308772)</f>
-        <v>0.131626442308772</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
+        <v>0.0965041812357258</v>
       </c>
       <c r="D6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
+        <v>0.0965041812357258</v>
       </c>
       <c r="E6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
+        <v>0.0965041812357258</v>
       </c>
       <c r="F6" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
@@ -1998,8 +1998,8 @@
         <v>1</v>
       </c>
       <c r="P6" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),185)</f>
-        <v>185</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),136)</f>
+        <v>136</v>
       </c>
       <c r="Q6" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2043,16 +2043,16 @@
         <v>0.0830536456103754</v>
       </c>
       <c r="C7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.113191682697692)</f>
-        <v>0.113191682697692</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
+        <v>0.091115822090457</v>
       </c>
       <c r="D7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
+        <v>0.091115822090457</v>
       </c>
       <c r="E7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
+        <v>0.091115822090457</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
@@ -2095,8 +2095,8 @@
         <v>1</v>
       </c>
       <c r="P7" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),967)</f>
-        <v>967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),778)</f>
+        <v>778</v>
       </c>
       <c r="Q7" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),69628)</f>
@@ -2140,16 +2140,16 @@
         <v>0.078155341572415</v>
       </c>
       <c r="C8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.140291242703435)</f>
-        <v>0.140291242703435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
+        <v>0.0988673086160884</v>
       </c>
       <c r="D8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
+        <v>0.0988673086160884</v>
       </c>
       <c r="E8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
+        <v>0.0988673086160884</v>
       </c>
       <c r="F8" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
@@ -2192,8 +2192,8 @@
         <v>1</v>
       </c>
       <c r="P8" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),73)</f>
-        <v>73</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),51)</f>
+        <v>51</v>
       </c>
       <c r="Q8" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2237,16 +2237,16 @@
         <v>0.0802492777307454</v>
       </c>
       <c r="C9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.1172579449618)</f>
-        <v>0.1172579449618</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
+        <v>0.0925855001410971</v>
       </c>
       <c r="D9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
+        <v>0.0925855001410971</v>
       </c>
       <c r="E9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
+        <v>0.0925855001410971</v>
       </c>
       <c r="F9" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
@@ -2289,8 +2289,8 @@
         <v>1</v>
       </c>
       <c r="P9" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),86)</f>
-        <v>86</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),68)</f>
+        <v>68</v>
       </c>
       <c r="Q9" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2625,16 +2625,16 @@
         <v>0.0771892846953241</v>
       </c>
       <c r="C13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.150917868351435)</f>
-        <v>0.150917868351435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
+        <v>0.101765479247361</v>
       </c>
       <c r="D13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
+        <v>0.101765479247361</v>
       </c>
       <c r="E13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
+        <v>0.101765479247361</v>
       </c>
       <c r="F13" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
@@ -2677,8 +2677,8 @@
         <v>1</v>
       </c>
       <c r="P13" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),54)</f>
-        <v>54</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37)</f>
+        <v>37</v>
       </c>
       <c r="Q13" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2722,16 +2722,16 @@
         <v>0.0787292505395418</v>
       </c>
       <c r="C14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.13397824406504)</f>
-        <v>0.13397824406504</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
+        <v>0.0971455817147079</v>
       </c>
       <c r="D14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
+        <v>0.0971455817147079</v>
       </c>
       <c r="E14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
+        <v>0.0971455817147079</v>
       </c>
       <c r="F14" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
@@ -2774,8 +2774,8 @@
         <v>1</v>
       </c>
       <c r="P14" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),258)</f>
-        <v>258</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),187)</f>
+        <v>187</v>
       </c>
       <c r="Q14" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2819,16 +2819,16 @@
         <v>0.0826992607152812</v>
       </c>
       <c r="C15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0903081321319072)</f>
-        <v>0.0903081321319072</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
+        <v>0.0852355511874899</v>
       </c>
       <c r="D15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
+        <v>0.0852355511874899</v>
       </c>
       <c r="E15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
+        <v>0.0852355511874899</v>
       </c>
       <c r="F15" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
@@ -2871,8 +2871,8 @@
         <v>1</v>
       </c>
       <c r="P15" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),62)</f>
-        <v>62</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),58)</f>
+        <v>58</v>
       </c>
       <c r="Q15" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3110,16 +3110,16 @@
         <v>0.0822850273487674</v>
       </c>
       <c r="C18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948646991635592)</f>
-        <v>0.0948646991635592</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
+        <v>0.0864782512870313</v>
       </c>
       <c r="D18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
+        <v>0.0864782512870313</v>
       </c>
       <c r="E18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
+        <v>0.0864782512870313</v>
       </c>
       <c r="F18" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
@@ -3162,8 +3162,8 @@
         <v>1</v>
       </c>
       <c r="P18" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9)</f>
-        <v>9</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8)</f>
+        <v>8</v>
       </c>
       <c r="Q18" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3207,16 +3207,16 @@
         <v>0.0822848847558399</v>
       </c>
       <c r="C19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948662676857615)</f>
-        <v>0.0948662676857615</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
+        <v>0.0864786790658138</v>
       </c>
       <c r="D19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
+        <v>0.0864786790658138</v>
       </c>
       <c r="E19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
+        <v>0.0864786790658138</v>
       </c>
       <c r="F19" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
@@ -3259,8 +3259,8 @@
         <v>1</v>
       </c>
       <c r="P19" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19)</f>
-        <v>19</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18)</f>
+        <v>18</v>
       </c>
       <c r="Q19" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3304,16 +3304,16 @@
         <v>0.0822852002059122</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948627977349655)</f>
-        <v>0.0948627977349655</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
+        <v>0.0864777327155967</v>
       </c>
       <c r="D20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
+        <v>0.0864777327155967</v>
       </c>
       <c r="E20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
+        <v>0.0864777327155967</v>
       </c>
       <c r="F20" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
@@ -3356,8 +3356,8 @@
         <v>1</v>
       </c>
       <c r="P20" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5)</f>
-        <v>5</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4)</f>
+        <v>4</v>
       </c>
       <c r="Q20" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3401,16 +3401,16 @@
         <v>0.082284103832348</v>
       </c>
       <c r="C21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948748578441723)</f>
-        <v>0.0948748578441723</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
+        <v>0.0864810218362894</v>
       </c>
       <c r="D21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
+        <v>0.0864810218362894</v>
       </c>
       <c r="E21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
+        <v>0.0864810218362894</v>
       </c>
       <c r="F21" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
@@ -3498,16 +3498,16 @@
         <v>0.101848800284409</v>
       </c>
       <c r="C22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955604631711142)</f>
-        <v>0.0955604631711142</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
+        <v>0.0837602978170431</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
+        <v>0.0837602978170431</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
+        <v>0.0837602978170431</v>
       </c>
       <c r="F22" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="P22" s="7" t="n">
         <f aca="false">SUM(P5:P21)</f>
-        <v>1757</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3757,16 +3757,16 @@
         <v>0.0295134514379623</v>
       </c>
       <c r="C30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.675352034182415)</f>
-        <v>0.675352034182415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
+        <v>0.244792979019447</v>
       </c>
       <c r="D30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
+        <v>0.244792979019447</v>
       </c>
       <c r="E30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
+        <v>0.244792979019447</v>
       </c>
       <c r="F30" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
@@ -4198,16 +4198,16 @@
         <v>0.0779725990367327</v>
       </c>
       <c r="C40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.14230141059594)</f>
-        <v>0.14230141059594</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
+        <v>0.0994155362231353</v>
       </c>
       <c r="D40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
+        <v>0.0994155362231353</v>
       </c>
       <c r="E40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
+        <v>0.0994155362231353</v>
       </c>
       <c r="F40" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
@@ -4250,8 +4250,8 @@
         <v>1</v>
       </c>
       <c r="P40" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),104)</f>
-        <v>104</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),73)</f>
+        <v>73</v>
       </c>
       <c r="Q40" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4295,16 +4295,16 @@
         <v>0.0824116289014618</v>
       </c>
       <c r="C41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.121277469433113)</f>
-        <v>0.121277469433113</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
+        <v>0.0933072507565163</v>
       </c>
       <c r="D41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
+        <v>0.0933072507565163</v>
       </c>
       <c r="E41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
+        <v>0.0933072507565163</v>
       </c>
       <c r="F41" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
@@ -4347,8 +4347,8 @@
         <v>1</v>
       </c>
       <c r="P41" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),540)</f>
-        <v>540</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),415)</f>
+        <v>415</v>
       </c>
       <c r="Q41" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),36760)</f>
@@ -4392,16 +4392,16 @@
         <v>0.0770946445386376</v>
       </c>
       <c r="C42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.151958910074986)</f>
-        <v>0.151958910074986</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
+        <v>0.10204939971742</v>
       </c>
       <c r="D42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
+        <v>0.10204939971742</v>
       </c>
       <c r="E42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
+        <v>0.10204939971742</v>
       </c>
       <c r="F42" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
@@ -4444,8 +4444,8 @@
         <v>1</v>
       </c>
       <c r="P42" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),41)</f>
-        <v>41</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28)</f>
+        <v>28</v>
       </c>
       <c r="Q42" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4489,16 +4489,16 @@
         <v>0.0793823941427303</v>
       </c>
       <c r="C43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.126793664429966)</f>
-        <v>0.126793664429966</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
+        <v>0.0951861509051423</v>
       </c>
       <c r="D43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
+        <v>0.0951861509051423</v>
       </c>
       <c r="E43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
+        <v>0.0951861509051423</v>
       </c>
       <c r="F43" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
@@ -4541,8 +4541,8 @@
         <v>1</v>
       </c>
       <c r="P43" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),49)</f>
-        <v>49</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37)</f>
+        <v>37</v>
       </c>
       <c r="Q43" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4877,16 +4877,16 @@
         <v>0.0758238813821944</v>
       </c>
       <c r="C47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.165937304795862)</f>
-        <v>0.165937304795862</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
+        <v>0.10586168918675</v>
       </c>
       <c r="D47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
+        <v>0.10586168918675</v>
       </c>
       <c r="E47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
+        <v>0.10586168918675</v>
       </c>
       <c r="F47" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
@@ -4929,8 +4929,8 @@
         <v>1</v>
       </c>
       <c r="P47" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31)</f>
-        <v>31</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),20)</f>
+        <v>20</v>
       </c>
       <c r="Q47" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4974,16 +4974,16 @@
         <v>0.0776565294661689</v>
       </c>
       <c r="C48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.145778175872141)</f>
-        <v>0.145778175872141</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
+        <v>0.100363744934826</v>
       </c>
       <c r="D48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
+        <v>0.100363744934826</v>
       </c>
       <c r="E48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
+        <v>0.100363744934826</v>
       </c>
       <c r="F48" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
@@ -5026,8 +5026,8 @@
         <v>1</v>
       </c>
       <c r="P48" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),146)</f>
-        <v>146</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),101)</f>
+        <v>101</v>
       </c>
       <c r="Q48" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5071,16 +5071,16 @@
         <v>0.0824962815446097</v>
       </c>
       <c r="C49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925409030092935)</f>
-        <v>0.0925409030092935</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
+        <v>0.0858444886995043</v>
       </c>
       <c r="D49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
+        <v>0.0858444886995043</v>
       </c>
       <c r="E49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
+        <v>0.0858444886995043</v>
       </c>
       <c r="F49" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
@@ -5123,8 +5123,8 @@
         <v>1</v>
       </c>
       <c r="P49" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),33)</f>
-        <v>33</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31)</f>
+        <v>31</v>
       </c>
       <c r="Q49" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5362,16 +5362,16 @@
         <v>0.0819169643322097</v>
       </c>
       <c r="C52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0989133923456932)</f>
-        <v>0.0989133923456932</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
+        <v>0.0875824403367042</v>
       </c>
       <c r="D52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
+        <v>0.0875824403367042</v>
       </c>
       <c r="E52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
+        <v>0.0875824403367042</v>
       </c>
       <c r="F52" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
@@ -5459,16 +5459,16 @@
         <v>0.0819175760181933</v>
       </c>
       <c r="C53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0989066637998739)</f>
-        <v>0.0989066637998739</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
+        <v>0.0875806052787535</v>
       </c>
       <c r="D53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
+        <v>0.0875806052787535</v>
       </c>
       <c r="E53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
+        <v>0.0875806052787535</v>
       </c>
       <c r="F53" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
@@ -5511,8 +5511,8 @@
         <v>1</v>
       </c>
       <c r="P53" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11)</f>
-        <v>11</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10)</f>
+        <v>10</v>
       </c>
       <c r="Q53" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5556,16 +5556,16 @@
         <v>0.0819180495097435</v>
       </c>
       <c r="C54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0989014553928212)</f>
-        <v>0.0989014553928212</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
+        <v>0.0875791848041027</v>
       </c>
       <c r="D54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
+        <v>0.0875791848041027</v>
       </c>
       <c r="E54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
+        <v>0.0875791848041027</v>
       </c>
       <c r="F54" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
@@ -5608,8 +5608,8 @@
         <v>1</v>
       </c>
       <c r="P54" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3)</f>
-        <v>3</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2)</f>
+        <v>2</v>
       </c>
       <c r="Q54" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5653,16 +5653,16 @@
         <v>0.0819179890740179</v>
       </c>
       <c r="C55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0989021201858035)</f>
-        <v>0.0989021201858035</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
+        <v>0.0875793661112797</v>
       </c>
       <c r="D55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
+        <v>0.0875793661112797</v>
       </c>
       <c r="E55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
+        <v>0.0875793661112797</v>
       </c>
       <c r="F55" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
@@ -5750,16 +5750,16 @@
         <v>0.1015098507676</v>
       </c>
       <c r="C56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0996205288380497)</f>
-        <v>0.0996205288380497</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
+        <v>0.0848631221776276</v>
       </c>
       <c r="D56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
+        <v>0.0848631221776276</v>
       </c>
       <c r="E56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
+        <v>0.0848631221776276</v>
       </c>
       <c r="F56" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="P56" s="7" t="n">
         <f aca="false">SUM(P39:P55)</f>
-        <v>985</v>
+        <v>744</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6009,16 +6009,16 @@
         <v>0.0269650818628408</v>
       </c>
       <c r="C64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.703384099508751)</f>
-        <v>0.703384099508751</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
+        <v>0.252438087744811</v>
       </c>
       <c r="D64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
+        <v>0.252438087744811</v>
       </c>
       <c r="E64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
+        <v>0.252438087744811</v>
       </c>
       <c r="F64" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
@@ -8104,11 +8104,11 @@
       </c>
       <c r="E76" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1757</v>
+        <v>1384</v>
       </c>
       <c r="I76" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>985</v>
+        <v>744</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Recargas: estacionalidad por rubro con fuentes y Excel renombrados a Aprovechamiento
- Automotor: enero y diciembre 12 %, noviembre y febrero de transición (ITV Córdoba, RTO Mendoza)
- Edificios, educación, hoteles, salud y supermercados con meses preferidos y vedados de sus pliegos, cámaras y
  manuales (peso a = 1/3, criterio); industrias sin estacionalidad
- Dimensionamiento_* pasa a Aprovechamiento_* en los archivos y en todas las referencias (Links, notas y Word)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Recargas.xlsx
+++ b/salida/Recargas.xlsx
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Qué se importa</t>
   </si>
   <si>
-    <t xml:space="preserve">Dimensionamiento Recargas Planta Comercial</t>
+    <t xml:space="preserve">Aprovechamiento Recargas Planta Comercial</t>
   </si>
   <si>
     <t xml:space="preserve">PEGAR ACÁ EL LINK DEL GOOGLE SHEET</t>
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Lo que trae la hoja Importados</t>
   </si>
   <si>
-    <t xml:space="preserve">Dimensionamiento Recargas Planta Industrial</t>
+    <t xml:space="preserve">Aprovechamiento Recargas Planta Industrial</t>
   </si>
   <si>
     <t xml:space="preserve">Recargas — logística de las dos plantas (mes pico de 2035)</t>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Stock de sustitutos (u)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dimensionamiento, paso 3</t>
+    <t xml:space="preserve">Aprovechamiento, paso 3</t>
   </si>
   <si>
     <t xml:space="preserve">Paradas por día</t>
@@ -275,7 +275,7 @@
     <t xml:space="preserve">Pasillo compartido por dos filas</t>
   </si>
   <si>
-    <t xml:space="preserve">Importados de los Dimensionamientos de recargas (IMPORTRANGE; el link va en la hoja Links)</t>
+    <t xml:space="preserve">Importados de los Aprovechamientos de recargas (IMPORTRANGE; el link va en la hoja Links)</t>
   </si>
   <si>
     <t xml:space="preserve">Planta comercial</t>
@@ -1260,11 +1260,11 @@
       </c>
       <c r="B6" s="8" t="str">
         <f aca="false">Cálculo!B6</f>
-        <v>Ene</v>
+        <v>Dic</v>
       </c>
       <c r="C6" s="8" t="str">
         <f aca="false">Cálculo!C6</f>
-        <v>Ene</v>
+        <v>Dic</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>18</v>
@@ -1276,11 +1276,11 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">Cálculo!F30</f>
-        <v>1050.21469306323</v>
+        <v>1061.94364471736</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">Cálculo!I30</f>
-        <v>544.079465849846</v>
+        <v>552.297705704186</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>20</v>
@@ -1292,11 +1292,11 @@
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Cálculo!G30</f>
-        <v>397.522456343171</v>
+        <v>409.324808263162</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">Cálculo!J30</f>
-        <v>204.786911560761</v>
+        <v>213.042982501654</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>20</v>
@@ -1308,11 +1308,11 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1384</v>
+        <v>1498</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>744</v>
+        <v>785</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>23</v>
@@ -1324,11 +1324,11 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">Cálculo!E44</f>
-        <v>202.933635977327</v>
+        <v>203.873824185969</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">Cálculo!I44</f>
-        <v>104.932589629389</v>
+        <v>105.685449564868</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>25</v>
@@ -1372,11 +1372,11 @@
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">Cálculo!B64</f>
-        <v>0.884975066104527</v>
+        <v>0.890469451056304</v>
       </c>
       <c r="C13" s="10" t="n">
         <f aca="false">Cálculo!C64</f>
-        <v>0.801437510401173</v>
+        <v>0.808620119744484</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Cálculo!E74</f>
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Cálculo!I74</f>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">Cálculo!E75</f>
-        <v>127.2</v>
+        <v>132</v>
       </c>
       <c r="C15" s="11" t="n">
         <f aca="false">Cálculo!I75</f>
@@ -1420,11 +1420,11 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Cálculo!E77</f>
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">Cálculo!I77</f>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>31</v>
@@ -1845,52 +1845,52 @@
         <v>109</v>
       </c>
       <c r="B5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E55:P72"")"),0.119933202334914)</f>
-        <v>0.119933202334914</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""parametros_recargas!E55:P72"")"),0.119877958433184)</f>
+        <v>0.119877958433184</v>
       </c>
       <c r="C5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0954780457654631)</f>
+        <v>0.0954780457654631</v>
       </c>
       <c r="D5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711264175844748)</f>
+        <v>0.0711264175844748</v>
       </c>
       <c r="E5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711264175844748)</f>
+        <v>0.0711264175844748</v>
       </c>
       <c r="F5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711747020712071)</f>
+        <v>0.0711747020712071</v>
       </c>
       <c r="G5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711747020712071)</f>
+        <v>0.0711747020712071</v>
       </c>
       <c r="H5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0710911890912281)</f>
+        <v>0.0710911890912281</v>
       </c>
       <c r="I5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711747020712071)</f>
+        <v>0.0711747020712071</v>
       </c>
       <c r="J5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711681740744643)</f>
+        <v>0.0711681740744643</v>
       </c>
       <c r="K5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711681740744643)</f>
+        <v>0.0711681740744643</v>
       </c>
       <c r="L5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760133595330172)</f>
-        <v>0.0760133595330172</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955198022554526)</f>
+        <v>0.0955198022554526</v>
       </c>
       <c r="M5" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119933202334914)</f>
-        <v>0.119933202334914</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119919714923173)</f>
+        <v>0.119919714923173</v>
       </c>
       <c r="N5" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""datos_base!K2:K18"")"),108842.626397553)</f>
@@ -1942,52 +1942,52 @@
         <v>110</v>
       </c>
       <c r="B6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0599939658092665)</f>
+        <v>0.0599939658092665</v>
       </c>
       <c r="C6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
-        <v>0.0965041812357258</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0599939658092665)</f>
+        <v>0.0599939658092665</v>
       </c>
       <c r="D6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
-        <v>0.0965041812357258</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0823418371052526)</f>
+        <v>0.0823418371052526</v>
       </c>
       <c r="E6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0965041812357258)</f>
-        <v>0.0965041812357258</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0958991878073455)</f>
+        <v>0.0958991878073455</v>
       </c>
       <c r="F6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10379748734495)</f>
+        <v>0.10379748734495</v>
       </c>
       <c r="G6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.102624553445736)</f>
+        <v>0.102624553445736</v>
       </c>
       <c r="H6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0742053590647476)</f>
+        <v>0.0742053590647476</v>
       </c>
       <c r="I6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0870020477881409)</f>
+        <v>0.0870020477881409</v>
       </c>
       <c r="J6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0871913152503224)</f>
+        <v>0.0871913152503224</v>
       </c>
       <c r="K6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0871913152503224)</f>
+        <v>0.0871913152503224</v>
       </c>
       <c r="L6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0792930157127176)</f>
+        <v>0.0792930157127176</v>
       </c>
       <c r="M6" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789430506992025)</f>
-        <v>0.0789430506992025</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0804659496119317)</f>
+        <v>0.0804659496119317</v>
       </c>
       <c r="N6" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9216.54014430766)</f>
@@ -1998,8 +1998,8 @@
         <v>1</v>
       </c>
       <c r="P6" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),136)</f>
-        <v>136</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),146)</f>
+        <v>146</v>
       </c>
       <c r="Q6" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2039,52 +2039,52 @@
         <v>111</v>
       </c>
       <c r="B7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0830536456103754)</f>
-        <v>0.0830536456103754</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0667556231939292)</f>
+        <v>0.0667556231939292</v>
       </c>
       <c r="C7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
-        <v>0.091115822090457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0651024266252983)</f>
+        <v>0.0651024266252983</v>
       </c>
       <c r="D7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
-        <v>0.091115822090457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0817858344236914)</f>
+        <v>0.0817858344236914</v>
       </c>
       <c r="E7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.091115822090457)</f>
-        <v>0.091115822090457</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0997196200427302)</f>
+        <v>0.0997196200427302</v>
       </c>
       <c r="F7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100089910575874)</f>
+        <v>0.100089910575874</v>
       </c>
       <c r="G7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988243995547109)</f>
+        <v>0.0988243995547109</v>
       </c>
       <c r="H7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0797892781627565)</f>
+        <v>0.0797892781627565</v>
       </c>
       <c r="I7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795925746996675)</f>
+        <v>0.0795925746996675</v>
       </c>
       <c r="J7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0807139532651435)</f>
+        <v>0.0807139532651435</v>
       </c>
       <c r="K7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0807139532651435)</f>
+        <v>0.0807139532651435</v>
       </c>
       <c r="L7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0800778917868397)</f>
-        <v>0.0800778917868397</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819968593006307)</f>
+        <v>0.0819968593006307</v>
       </c>
       <c r="M7" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0830536456103754)</f>
-        <v>0.0830536456103754</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0849155668904246)</f>
+        <v>0.0849155668904246</v>
       </c>
       <c r="N7" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),56059.2707104735)</f>
@@ -2095,8 +2095,8 @@
         <v>1</v>
       </c>
       <c r="P7" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),778)</f>
-        <v>778</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),855)</f>
+        <v>855</v>
       </c>
       <c r="Q7" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),69628)</f>
@@ -2136,52 +2136,52 @@
         <v>112</v>
       </c>
       <c r="B8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.064612341974598)</f>
+        <v>0.064612341974598</v>
       </c>
       <c r="C8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
-        <v>0.0988673086160884</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.064612341974598)</f>
+        <v>0.064612341974598</v>
       </c>
       <c r="D8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
-        <v>0.0988673086160884</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0831857089056497)</f>
+        <v>0.0831857089056497</v>
       </c>
       <c r="E8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0988673086160884)</f>
-        <v>0.0988673086160884</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101329540689849)</f>
+        <v>0.101329540689849</v>
       </c>
       <c r="F8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10227719847342)</f>
+        <v>0.10227719847342</v>
       </c>
       <c r="G8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993233886074831)</f>
+        <v>0.0993233886074831</v>
       </c>
       <c r="H8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078066397641533)</f>
+        <v>0.078066397641533</v>
       </c>
       <c r="I8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078743869594065)</f>
+        <v>0.078743869594065</v>
       </c>
       <c r="J8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081697679460002)</f>
+        <v>0.081697679460002</v>
       </c>
       <c r="K8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081697679460002)</f>
+        <v>0.081697679460002</v>
       </c>
       <c r="L8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0807500216764314)</f>
+        <v>0.0807500216764314</v>
       </c>
       <c r="M8" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078155341572415)</f>
-        <v>0.078155341572415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837038315423683)</f>
+        <v>0.0837038315423683</v>
       </c>
       <c r="N8" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3319.32790518283)</f>
@@ -2192,8 +2192,8 @@
         <v>1</v>
       </c>
       <c r="P8" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),51)</f>
-        <v>51</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),53)</f>
+        <v>53</v>
       </c>
       <c r="Q8" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2233,52 +2233,52 @@
         <v>113</v>
       </c>
       <c r="B9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0670768247329043)</f>
+        <v>0.0670768247329043</v>
       </c>
       <c r="C9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
-        <v>0.0925855001410971</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0670768247329043)</f>
+        <v>0.0670768247329043</v>
       </c>
       <c r="D9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
-        <v>0.0925855001410971</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0827868661277296)</f>
+        <v>0.0827868661277296</v>
       </c>
       <c r="E9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0925855001410971)</f>
-        <v>0.0925855001410971</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0993493196011858)</f>
+        <v>0.0993493196011858</v>
       </c>
       <c r="F9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0999705290370024)</f>
+        <v>0.0999705290370024</v>
       </c>
       <c r="G9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0970461916480882)</f>
+        <v>0.0970461916480882</v>
       </c>
       <c r="H9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788828581851096)</f>
+        <v>0.0788828581851096</v>
       </c>
       <c r="I9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0790330223001652)</f>
+        <v>0.0790330223001652</v>
       </c>
       <c r="J9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0817739112794073)</f>
+        <v>0.0817739112794073</v>
       </c>
       <c r="K9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0817739112794073)</f>
+        <v>0.0817739112794073</v>
       </c>
       <c r="L9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0811527018435908)</f>
+        <v>0.0811527018435908</v>
       </c>
       <c r="M9" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0802492777307454)</f>
-        <v>0.0802492777307454</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.084077039232505)</f>
+        <v>0.084077039232505</v>
       </c>
       <c r="N9" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4686.14321768856)</f>
@@ -2289,8 +2289,8 @@
         <v>1</v>
       </c>
       <c r="P9" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),68)</f>
-        <v>68</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),73)</f>
+        <v>73</v>
       </c>
       <c r="Q9" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2621,52 +2621,52 @@
         <v>117</v>
       </c>
       <c r="B13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0695355190499093)</f>
+        <v>0.0695355190499093</v>
       </c>
       <c r="C13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
-        <v>0.101765479247361</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0695355190499093)</f>
+        <v>0.0695355190499093</v>
       </c>
       <c r="D13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
-        <v>0.101765479247361</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0838248196490894)</f>
+        <v>0.0838248196490894</v>
       </c>
       <c r="E13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101765479247361)</f>
-        <v>0.101765479247361</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948339806026096)</f>
+        <v>0.0948339806026096</v>
       </c>
       <c r="F13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0972184056200527)</f>
+        <v>0.0972184056200527</v>
       </c>
       <c r="G13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0952240073446056)</f>
+        <v>0.0952240073446056</v>
       </c>
       <c r="H13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0780009399043672)</f>
+        <v>0.0780009399043672</v>
       </c>
       <c r="I13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0813247334874215)</f>
+        <v>0.0813247334874215</v>
       </c>
       <c r="J13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833191317628686)</f>
+        <v>0.0833191317628686</v>
       </c>
       <c r="K13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833191317628686)</f>
+        <v>0.0833191317628686</v>
       </c>
       <c r="L13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809347067454255)</f>
+        <v>0.0809347067454255</v>
       </c>
       <c r="M13" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771892846953241)</f>
-        <v>0.0771892846953241</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0829291050208727)</f>
+        <v>0.0829291050208727</v>
       </c>
       <c r="N13" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2310.99407344162)</f>
@@ -2677,8 +2677,8 @@
         <v>1</v>
       </c>
       <c r="P13" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37)</f>
-        <v>37</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),35)</f>
+        <v>35</v>
       </c>
       <c r="Q13" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2718,52 +2718,52 @@
         <v>118</v>
       </c>
       <c r="B14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0616150736413202)</f>
+        <v>0.0616150736413202</v>
       </c>
       <c r="C14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
-        <v>0.0971455817147079</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0616150736413202)</f>
+        <v>0.0616150736413202</v>
       </c>
       <c r="D14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
-        <v>0.0971455817147079</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0829453490803136)</f>
+        <v>0.0829453490803136</v>
       </c>
       <c r="E14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0971455817147079)</f>
-        <v>0.0971455817147079</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.103007646651263)</f>
+        <v>0.103007646651263</v>
       </c>
       <c r="F14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.103425871740429)</f>
+        <v>0.103425871740429</v>
       </c>
       <c r="G14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.102109899624234)</f>
+        <v>0.102109899624234</v>
       </c>
       <c r="H14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0801282894274162)</f>
+        <v>0.0801282894274162</v>
       </c>
       <c r="I14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.079881877158212)</f>
+        <v>0.079881877158212</v>
       </c>
       <c r="J14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081197849274407)</f>
+        <v>0.081197849274407</v>
       </c>
       <c r="K14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081197849274407)</f>
+        <v>0.081197849274407</v>
       </c>
       <c r="L14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.080779624185241)</f>
+        <v>0.080779624185241</v>
       </c>
       <c r="M14" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0787292505395418)</f>
-        <v>0.0787292505395418</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082095596301436)</f>
+        <v>0.082095596301436</v>
       </c>
       <c r="N14" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12606.7299522508)</f>
@@ -2774,8 +2774,8 @@
         <v>1</v>
       </c>
       <c r="P14" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),187)</f>
-        <v>187</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),199)</f>
+        <v>199</v>
       </c>
       <c r="Q14" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2815,52 +2815,52 @@
         <v>119</v>
       </c>
       <c r="B15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761848278176029)</f>
+        <v>0.0761848278176029</v>
       </c>
       <c r="C15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
-        <v>0.0852355511874899</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761848278176029)</f>
+        <v>0.0761848278176029</v>
       </c>
       <c r="D15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
-        <v>0.0852355511874899</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826686065765467)</f>
+        <v>0.0826686065765467</v>
       </c>
       <c r="E15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0852355511874899)</f>
-        <v>0.0852355511874899</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0916518877640263)</f>
+        <v>0.0916518877640263</v>
       </c>
       <c r="F15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0931955183643168)</f>
+        <v>0.0931955183643168</v>
       </c>
       <c r="G15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0888541224858191)</f>
+        <v>0.0888541224858191</v>
       </c>
       <c r="H15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0784912986070083)</f>
+        <v>0.0784912986070083</v>
       </c>
       <c r="I15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795725784486681)</f>
+        <v>0.0795725784486681</v>
       </c>
       <c r="J15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0829855493601231)</f>
+        <v>0.0829855493601231</v>
       </c>
       <c r="K15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0829855493601231)</f>
+        <v>0.0829855493601231</v>
       </c>
       <c r="L15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0814419187598326)</f>
+        <v>0.0814419187598326</v>
       </c>
       <c r="M15" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826992607152812)</f>
-        <v>0.0826992607152812</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0857833146383303)</f>
+        <v>0.0857833146383303</v>
       </c>
       <c r="N15" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4308.38387982745)</f>
@@ -2871,8 +2871,8 @@
         <v>1</v>
       </c>
       <c r="P15" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),58)</f>
-        <v>58</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),64)</f>
+        <v>64</v>
       </c>
       <c r="Q15" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -2912,12 +2912,12 @@
         <v>120</v>
       </c>
       <c r="B16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0890943915723948)</f>
+        <v>0.0890943915723948</v>
       </c>
       <c r="C16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0890943915723948)</f>
+        <v>0.0890943915723948</v>
       </c>
       <c r="D16" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -2932,16 +2932,16 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="G16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0775722750942719)</f>
+        <v>0.0775722750942719</v>
       </c>
       <c r="H16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0775722750942719)</f>
+        <v>0.0775722750942719</v>
       </c>
       <c r="I16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0775722750942719)</f>
+        <v>0.0775722750942719</v>
       </c>
       <c r="J16" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -2956,8 +2956,8 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="M16" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0890943915723948)</f>
+        <v>0.0890943915723948</v>
       </c>
       <c r="N16" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),705.316446113659)</f>
@@ -2968,8 +2968,8 @@
         <v>1</v>
       </c>
       <c r="P16" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10)</f>
-        <v>10</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11)</f>
+        <v>11</v>
       </c>
       <c r="Q16" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3106,52 +3106,52 @@
         <v>122</v>
       </c>
       <c r="B18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741713639081832)</f>
+        <v>0.0741713639081832</v>
       </c>
       <c r="C18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
-        <v>0.0864782512870313</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741713639081832)</f>
+        <v>0.0741713639081832</v>
       </c>
       <c r="D18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
-        <v>0.0864782512870313</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826308825789044)</f>
+        <v>0.0826308825789044</v>
       </c>
       <c r="E18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864782512870313)</f>
-        <v>0.0864782512870313</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0938477438743188)</f>
+        <v>0.0938477438743188</v>
       </c>
       <c r="F18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0943031990696216)</f>
+        <v>0.0943031990696216</v>
       </c>
       <c r="G18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905972862319092)</f>
+        <v>0.0905972862319092</v>
       </c>
       <c r="H18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782229570370311)</f>
+        <v>0.0782229570370311</v>
       </c>
       <c r="I18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788873099187785)</f>
+        <v>0.0788873099187785</v>
       </c>
       <c r="J18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825932227564908)</f>
+        <v>0.0825932227564908</v>
       </c>
       <c r="K18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825932227564908)</f>
+        <v>0.0825932227564908</v>
       </c>
       <c r="L18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082137767561188)</f>
+        <v>0.082137767561188</v>
       </c>
       <c r="M18" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822850273487674)</f>
-        <v>0.0822850273487674</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858436803989003)</f>
+        <v>0.0858436803989003</v>
       </c>
       <c r="N18" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),577.776131502584)</f>
@@ -3162,8 +3162,8 @@
         <v>1</v>
       </c>
       <c r="P18" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8)</f>
-        <v>8</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9)</f>
+        <v>9</v>
       </c>
       <c r="Q18" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3203,52 +3203,52 @@
         <v>123</v>
       </c>
       <c r="B19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741714575622674)</f>
+        <v>0.0741714575622674</v>
       </c>
       <c r="C19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
-        <v>0.0864786790658138</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741714575622674)</f>
+        <v>0.0741714575622674</v>
       </c>
       <c r="D19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
-        <v>0.0864786790658138</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08263095051887)</f>
+        <v>0.08263095051887</v>
       </c>
       <c r="E19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864786790658138)</f>
-        <v>0.0864786790658138</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0938477343304375)</f>
+        <v>0.0938477343304375</v>
       </c>
       <c r="F19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0943030721576538)</f>
+        <v>0.0943030721576538</v>
       </c>
       <c r="G19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905972613831472)</f>
+        <v>0.0905972613831472</v>
       </c>
       <c r="H19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782232108709845)</f>
+        <v>0.0782232108709845</v>
       </c>
       <c r="I19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788872954792544)</f>
+        <v>0.0788872954792544</v>
       </c>
       <c r="J19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082593106253761)</f>
+        <v>0.082593106253761</v>
       </c>
       <c r="K19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082593106253761)</f>
+        <v>0.082593106253761</v>
       </c>
       <c r="L19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0821377684265447)</f>
+        <v>0.0821377684265447</v>
       </c>
       <c r="M19" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822848847558399)</f>
-        <v>0.0822848847558399</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858435792010512)</f>
+        <v>0.0858435792010512</v>
       </c>
       <c r="N19" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1271.10748852936)</f>
@@ -3259,8 +3259,8 @@
         <v>1</v>
       </c>
       <c r="P19" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18)</f>
-        <v>18</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19)</f>
+        <v>19</v>
       </c>
       <c r="Q19" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3300,52 +3300,52 @@
         <v>124</v>
       </c>
       <c r="B20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741714711262728)</f>
+        <v>0.0741714711262728</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
-        <v>0.0864777327155967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741714711262728)</f>
+        <v>0.0741714711262728</v>
       </c>
       <c r="D20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
-        <v>0.0864777327155967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826308668449537)</f>
+        <v>0.0826308668449537</v>
       </c>
       <c r="E20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864777327155967)</f>
-        <v>0.0864777327155967</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0938479481909226)</f>
+        <v>0.0938479481909226</v>
       </c>
       <c r="F20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0943030828496681)</f>
+        <v>0.0943030828496681</v>
       </c>
       <c r="G20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905972288565807)</f>
+        <v>0.0905972288565807</v>
       </c>
       <c r="H20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782233613395939)</f>
+        <v>0.0782233613395939</v>
       </c>
       <c r="I20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788871138035579)</f>
+        <v>0.0788871138035579</v>
       </c>
       <c r="J20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825929677966453)</f>
+        <v>0.0825929677966453</v>
       </c>
       <c r="K20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825929677966453)</f>
+        <v>0.0825929677966453</v>
       </c>
       <c r="L20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0821378331378998)</f>
+        <v>0.0821378331378998</v>
       </c>
       <c r="M20" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0822852002059122)</f>
-        <v>0.0822852002059122</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858436871309872)</f>
+        <v>0.0858436871309872</v>
       </c>
       <c r="N20" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),277.332543143421)</f>
@@ -3356,8 +3356,8 @@
         <v>1</v>
       </c>
       <c r="P20" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4)</f>
-        <v>4</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5)</f>
+        <v>5</v>
       </c>
       <c r="Q20" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -3397,52 +3397,52 @@
         <v>125</v>
       </c>
       <c r="B21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741721346584101)</f>
+        <v>0.0741721346584101</v>
       </c>
       <c r="C21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
-        <v>0.0864810218362894</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0741721346584101)</f>
+        <v>0.0741721346584101</v>
       </c>
       <c r="D21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
-        <v>0.0864810218362894</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826312550911103)</f>
+        <v>0.0826312550911103</v>
       </c>
       <c r="E21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864810218362894)</f>
-        <v>0.0864810218362894</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0938475454254633)</f>
+        <v>0.0938475454254633</v>
       </c>
       <c r="F21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0943026800842088)</f>
+        <v>0.0943026800842088</v>
       </c>
       <c r="G21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0905968260911214)</f>
+        <v>0.0905968260911214</v>
       </c>
       <c r="H21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782234917229329)</f>
+        <v>0.0782234917229329</v>
       </c>
       <c r="I21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788869863240794)</f>
+        <v>0.0788869863240794</v>
       </c>
       <c r="J21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825928403171668)</f>
+        <v>0.0825928403171668</v>
       </c>
       <c r="K21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0825928403171668)</f>
+        <v>0.0825928403171668</v>
       </c>
       <c r="L21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0821377056584213)</f>
+        <v>0.0821377056584213</v>
       </c>
       <c r="M21" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082284103832348)</f>
-        <v>0.082284103832348</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858435596515087)</f>
+        <v>0.0858435596515087</v>
       </c>
       <c r="N21" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),184.888361725934)</f>
@@ -3494,52 +3494,52 @@
         <v>126</v>
       </c>
       <c r="B22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101848800284409)</f>
-        <v>0.101848800284409</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.094685974590863)</f>
+        <v>0.094685974590863</v>
       </c>
       <c r="C22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
-        <v>0.0837602978170431</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0813589828439731)</f>
+        <v>0.0813589828439731</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
-        <v>0.0837602978170431</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0763711312806997)</f>
+        <v>0.0763711312806997</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0837602978170431)</f>
-        <v>0.0837602978170431</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.084183445923961)</f>
+        <v>0.084183445923961</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0847815688752799)</f>
+        <v>0.0847815688752799</v>
       </c>
       <c r="G22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0840164331631308)</f>
+        <v>0.0840164331631308</v>
       </c>
       <c r="H22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0748812526033842)</f>
+        <v>0.0748812526033842</v>
       </c>
       <c r="I22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0755102802186843)</f>
+        <v>0.0755102802186843</v>
       </c>
       <c r="J22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761652663624608)</f>
+        <v>0.0761652663624608</v>
       </c>
       <c r="K22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761652663624608)</f>
+        <v>0.0761652663624608</v>
       </c>
       <c r="L22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0778602151400075)</f>
-        <v>0.0778602151400075</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0888941351580317)</f>
+        <v>0.0888941351580317</v>
       </c>
       <c r="M22" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101848800284409)</f>
-        <v>0.101848800284409</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.102986262617071)</f>
+        <v>0.102986262617071</v>
       </c>
       <c r="N22" s="7" t="n">
         <f aca="false">SUM(N5:N21)</f>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="P22" s="7" t="n">
         <f aca="false">SUM(P5:P21)</f>
-        <v>1384</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3651,44 +3651,44 @@
         <v>0.12</v>
       </c>
       <c r="C28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955555555555556)</f>
+        <v>0.0955555555555556</v>
       </c>
       <c r="D28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="E28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="F28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="G28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="H28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="I28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="J28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="K28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="L28" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955555555555556)</f>
+        <v>0.0955555555555556</v>
       </c>
       <c r="M28" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.12)</f>
@@ -3700,52 +3700,52 @@
         <v>102</v>
       </c>
       <c r="B29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0540540540540541)</f>
+        <v>0.0540540540540541</v>
       </c>
       <c r="C29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0540540540540541)</f>
+        <v>0.0540540540540541</v>
       </c>
       <c r="D29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="E29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="F29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="G29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="H29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="I29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="J29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="K29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="L29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="M29" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3753,52 +3753,52 @@
         <v>103</v>
       </c>
       <c r="B30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="C30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
-        <v>0.244792979019447</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="D30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
-        <v>0.244792979019447</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="E30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.244792979019447)</f>
-        <v>0.244792979019447</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="F30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="G30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="H30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0886075949367089)</f>
+        <v>0.0886075949367089</v>
       </c>
       <c r="I30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="J30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="K30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="L30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="M30" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0295134514379623)</f>
-        <v>0.0295134514379623</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,52 +3806,52 @@
         <v>104</v>
       </c>
       <c r="B31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="C31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="D31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="E31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="F31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="G31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="H31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="I31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="J31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="K31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="L31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="M31" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,12 +3912,12 @@
         <v>106</v>
       </c>
       <c r="B33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="C33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="D33" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -3932,16 +3932,16 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="G33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="H33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="I33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="J33" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -3956,8 +3956,8 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="M33" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3965,12 +3965,12 @@
         <v>107</v>
       </c>
       <c r="B34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="C34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="D34" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -3981,20 +3981,20 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="F34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="G34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="H34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="I34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="J34" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -4005,12 +4005,12 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="L34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="M34" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4097,52 +4097,52 @@
         <v>109</v>
       </c>
       <c r="B39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E55:P72"")"),0.119942566698092)</f>
-        <v>0.119942566698092</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""parametros_recargas!E55:P72"")"),0.119895289559294)</f>
+        <v>0.119895289559294</v>
       </c>
       <c r="C39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0954891339827875)</f>
+        <v>0.0954891339827875</v>
       </c>
       <c r="D39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.071124604952686)</f>
+        <v>0.071124604952686</v>
       </c>
       <c r="E39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.071124604952686)</f>
+        <v>0.071124604952686</v>
       </c>
       <c r="F39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711662314990906)</f>
+        <v>0.0711662314990906</v>
       </c>
       <c r="G39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711662314990906)</f>
+        <v>0.0711662314990906</v>
       </c>
       <c r="H39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0710984243903592)</f>
+        <v>0.0710984243903592</v>
       </c>
       <c r="I39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711662314990906)</f>
+        <v>0.0711662314990906</v>
       </c>
       <c r="J39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711585085070517)</f>
+        <v>0.0711585085070517</v>
       </c>
       <c r="K39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711585085070517)</f>
+        <v>0.0711585085070517</v>
       </c>
       <c r="L39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0760114866603815)</f>
-        <v>0.0760114866603815</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955230375371532)</f>
+        <v>0.0955230375371532</v>
       </c>
       <c r="M39" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119942566698092)</f>
-        <v>0.119942566698092</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.119929193113659)</f>
+        <v>0.119929193113659</v>
       </c>
       <c r="N39" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""datos_base!K2:K18"")"),56575.8368575054)</f>
@@ -4194,52 +4194,52 @@
         <v>110</v>
       </c>
       <c r="B40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0608346558815601)</f>
+        <v>0.0608346558815601</v>
       </c>
       <c r="C40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
-        <v>0.0994155362231353</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0608346558815601)</f>
+        <v>0.0608346558815601</v>
       </c>
       <c r="D40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
-        <v>0.0994155362231353</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082643351275423)</f>
+        <v>0.082643351275423</v>
       </c>
       <c r="E40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994155362231353)</f>
-        <v>0.0994155362231353</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0953382202836263)</f>
+        <v>0.0953382202836263</v>
       </c>
       <c r="F40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.103308847602848)</f>
+        <v>0.103308847602848</v>
       </c>
       <c r="G40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204440072004)</f>
+        <v>0.10204440072004</v>
       </c>
       <c r="H40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0745034484311485)</f>
+        <v>0.0745034484311485</v>
       </c>
       <c r="I40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0869418857625907)</f>
+        <v>0.0869418857625907</v>
       </c>
       <c r="J40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0870568354792096)</f>
+        <v>0.0870568354792096</v>
       </c>
       <c r="K40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0870568354792096)</f>
+        <v>0.0870568354792096</v>
       </c>
       <c r="L40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0790862081599875)</f>
+        <v>0.0790862081599875</v>
       </c>
       <c r="M40" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0779725990367327)</f>
-        <v>0.0779725990367327</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.080350655042796)</f>
+        <v>0.080350655042796</v>
       </c>
       <c r="N40" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4790.71011839089)</f>
@@ -4250,8 +4250,8 @@
         <v>1</v>
       </c>
       <c r="P40" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),73)</f>
-        <v>73</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),76)</f>
+        <v>76</v>
       </c>
       <c r="Q40" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4291,52 +4291,52 @@
         <v>111</v>
       </c>
       <c r="B41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824116289014618)</f>
-        <v>0.0824116289014618</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0669778155176287)</f>
+        <v>0.0669778155176287</v>
       </c>
       <c r="C41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
-        <v>0.0933072507565163</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0652614335824934)</f>
+        <v>0.0652614335824934</v>
       </c>
       <c r="D41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
-        <v>0.0933072507565163</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819248891202413)</f>
+        <v>0.0819248891202413</v>
       </c>
       <c r="E41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0933072507565163)</f>
-        <v>0.0933072507565163</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0996461832727322)</f>
+        <v>0.0996461832727322</v>
       </c>
       <c r="F41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100150076298148)</f>
+        <v>0.100150076298148</v>
       </c>
       <c r="G41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0987344570187928)</f>
+        <v>0.0987344570187928</v>
       </c>
       <c r="H41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0795692614778467)</f>
+        <v>0.0795692614778467</v>
       </c>
       <c r="I41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0794428932919701)</f>
+        <v>0.0794428932919701</v>
       </c>
       <c r="J41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0806840028465543)</f>
+        <v>0.0806840028465543</v>
       </c>
       <c r="K41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0806840028465543)</f>
+        <v>0.0806840028465543</v>
       </c>
       <c r="L41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793221414182182)</f>
-        <v>0.0793221414182182</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0818964917562743)</f>
+        <v>0.0818964917562743</v>
       </c>
       <c r="M41" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824116289014618)</f>
-        <v>0.0824116289014618</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0850284929707643)</f>
+        <v>0.0850284929707643</v>
       </c>
       <c r="N41" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),29139.3203107948)</f>
@@ -4347,8 +4347,8 @@
         <v>1</v>
       </c>
       <c r="P41" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),415)</f>
-        <v>415</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),446)</f>
+        <v>446</v>
       </c>
       <c r="Q41" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),36760)</f>
@@ -4388,52 +4388,52 @@
         <v>112</v>
       </c>
       <c r="B42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0656624516770873)</f>
+        <v>0.0656624516770873</v>
       </c>
       <c r="C42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
-        <v>0.10204939971742</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0656624516770873)</f>
+        <v>0.0656624516770873</v>
       </c>
       <c r="D42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
-        <v>0.10204939971742</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0834634227222184)</f>
+        <v>0.0834634227222184</v>
       </c>
       <c r="E42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10204939971742)</f>
-        <v>0.10204939971742</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100292059397134)</f>
+        <v>0.100292059397134</v>
       </c>
       <c r="F42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101604548245527)</f>
+        <v>0.101604548245527</v>
       </c>
       <c r="G42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0984624354955731)</f>
+        <v>0.0984624354955731</v>
       </c>
       <c r="H42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776078419879838)</f>
+        <v>0.0776078419879838</v>
       </c>
       <c r="I42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0788318405488818)</f>
+        <v>0.0788318405488818</v>
       </c>
       <c r="J42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819739532988352)</f>
+        <v>0.0819739532988352</v>
       </c>
       <c r="K42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819739532988352)</f>
+        <v>0.0819739532988352</v>
       </c>
       <c r="L42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0806614644504421)</f>
+        <v>0.0806614644504421</v>
       </c>
       <c r="M42" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0770946445386376)</f>
-        <v>0.0770946445386376</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0838035772003955)</f>
+        <v>0.0838035772003955</v>
       </c>
       <c r="N42" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1725.36955653994)</f>
@@ -4485,52 +4485,52 @@
         <v>113</v>
       </c>
       <c r="B43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0671288961017088)</f>
+        <v>0.0671288961017088</v>
       </c>
       <c r="C43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
-        <v>0.0951861509051423</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0671288961017088)</f>
+        <v>0.0671288961017088</v>
       </c>
       <c r="D43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
-        <v>0.0951861509051423</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082960331994099)</f>
+        <v>0.082960331994099</v>
       </c>
       <c r="E43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0951861509051423)</f>
-        <v>0.0951861509051423</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0994555948834204)</f>
+        <v>0.0994555948834204</v>
       </c>
       <c r="F43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100324801949947)</f>
+        <v>0.100324801949947</v>
       </c>
       <c r="G43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0970172977837637)</f>
+        <v>0.0970172977837637</v>
       </c>
       <c r="H43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0783455208911489)</f>
+        <v>0.0783455208911489</v>
       </c>
       <c r="I43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.078747564791717)</f>
+        <v>0.078747564791717</v>
       </c>
       <c r="J43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0818305013673391)</f>
+        <v>0.0818305013673391</v>
       </c>
       <c r="K43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0818305013673391)</f>
+        <v>0.0818305013673391</v>
       </c>
       <c r="L43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0809612943008125)</f>
+        <v>0.0809612943008125</v>
       </c>
       <c r="M43" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793823941427303)</f>
-        <v>0.0793823941427303</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0842687984669957)</f>
+        <v>0.0842687984669957</v>
       </c>
       <c r="N43" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2435.83311933763)</f>
@@ -4541,8 +4541,8 @@
         <v>1</v>
       </c>
       <c r="P43" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37)</f>
-        <v>37</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),39)</f>
+        <v>39</v>
       </c>
       <c r="Q43" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4873,52 +4873,52 @@
         <v>117</v>
       </c>
       <c r="B47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0693955234457278)</f>
+        <v>0.0693955234457278</v>
       </c>
       <c r="C47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
-        <v>0.10586168918675</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0693955234457278)</f>
+        <v>0.0693955234457278</v>
       </c>
       <c r="D47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
-        <v>0.10586168918675</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0840431757641277)</f>
+        <v>0.0840431757641277</v>
       </c>
       <c r="E47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10586168918675)</f>
-        <v>0.10586168918675</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0941202036639783)</f>
+        <v>0.0941202036639783</v>
       </c>
       <c r="F47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0974702272576739)</f>
+        <v>0.0974702272576739</v>
       </c>
       <c r="G47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.095318136848291)</f>
+        <v>0.095318136848291</v>
       </c>
       <c r="H47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076854716143931)</f>
+        <v>0.076854716143931</v>
       </c>
       <c r="I47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0818684177142039)</f>
+        <v>0.0818684177142039</v>
       </c>
       <c r="J47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0840205081235868)</f>
+        <v>0.0840205081235868</v>
       </c>
       <c r="K47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0840205081235868)</f>
+        <v>0.0840205081235868</v>
       </c>
       <c r="L47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0806704845298912)</f>
+        <v>0.0806704845298912</v>
       </c>
       <c r="M47" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758238813821944)</f>
-        <v>0.0758238813821944</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082822574939274)</f>
+        <v>0.082822574939274</v>
       </c>
       <c r="N47" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1201.24282190818)</f>
@@ -4929,8 +4929,8 @@
         <v>1</v>
       </c>
       <c r="P47" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),20)</f>
-        <v>20</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19)</f>
+        <v>19</v>
       </c>
       <c r="Q47" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -4970,52 +4970,52 @@
         <v>118</v>
       </c>
       <c r="B48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0623734752667158)</f>
+        <v>0.0623734752667158</v>
       </c>
       <c r="C48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
-        <v>0.100363744934826</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0623734752667158)</f>
+        <v>0.0623734752667158</v>
       </c>
       <c r="D48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
-        <v>0.100363744934826</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0832322896847601)</f>
+        <v>0.0832322896847601</v>
       </c>
       <c r="E48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.100363744934826)</f>
-        <v>0.100363744934826</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.102381291624983)</f>
+        <v>0.102381291624983</v>
       </c>
       <c r="F48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10297405651463)</f>
+        <v>0.10297405651463</v>
       </c>
       <c r="G48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.101541503044586)</f>
+        <v>0.101541503044586</v>
       </c>
       <c r="H48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0799321707959588)</f>
+        <v>0.0799321707959588</v>
       </c>
       <c r="I48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0798429000461445)</f>
+        <v>0.0798429000461445</v>
       </c>
       <c r="J48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081275453516189)</f>
+        <v>0.081275453516189</v>
       </c>
       <c r="K48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081275453516189)</f>
+        <v>0.081275453516189</v>
       </c>
       <c r="L48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0806826886265415)</f>
+        <v>0.0806826886265415</v>
       </c>
       <c r="M48" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776565294661689)</f>
-        <v>0.0776565294661689</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0821152420965861)</f>
+        <v>0.0821152420965861</v>
       </c>
       <c r="N48" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6552.91332717418)</f>
@@ -5026,8 +5026,8 @@
         <v>1</v>
       </c>
       <c r="P48" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),101)</f>
-        <v>101</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),103)</f>
+        <v>103</v>
       </c>
       <c r="Q48" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5067,52 +5067,52 @@
         <v>119</v>
       </c>
       <c r="B49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758899515991334)</f>
+        <v>0.0758899515991334</v>
       </c>
       <c r="C49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
-        <v>0.0858444886995043</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0758899515991334)</f>
+        <v>0.0758899515991334</v>
       </c>
       <c r="D49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
-        <v>0.0858444886995043</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.082635648810499)</f>
+        <v>0.082635648810499</v>
       </c>
       <c r="E49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0858444886995043)</f>
-        <v>0.0858444886995043</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0919604223371936)</f>
+        <v>0.0919604223371936</v>
       </c>
       <c r="F49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.094065383152575)</f>
+        <v>0.094065383152575</v>
       </c>
       <c r="G49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0890054041756688)</f>
+        <v>0.0890054041756688</v>
       </c>
       <c r="H49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0776256551320905)</f>
+        <v>0.0776256551320905</v>
       </c>
       <c r="I49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0793046888027784)</f>
+        <v>0.0793046888027784</v>
       </c>
       <c r="J49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0831932092611961)</f>
+        <v>0.0831932092611961</v>
       </c>
       <c r="K49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0831932092611961)</f>
+        <v>0.0831932092611961</v>
       </c>
       <c r="L49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810882484458147)</f>
+        <v>0.0810882484458147</v>
       </c>
       <c r="M49" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0824962815446097)</f>
-        <v>0.0824962815446097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0861482274227209)</f>
+        <v>0.0861482274227209</v>
       </c>
       <c r="N49" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2239.47576029921)</f>
@@ -5123,8 +5123,8 @@
         <v>1</v>
       </c>
       <c r="P49" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31)</f>
-        <v>31</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),34)</f>
+        <v>34</v>
       </c>
       <c r="Q49" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5164,12 +5164,12 @@
         <v>120</v>
       </c>
       <c r="B50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0909796762566006)</f>
+        <v>0.0909796762566006</v>
       </c>
       <c r="C50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0909796762566006)</f>
+        <v>0.0909796762566006</v>
       </c>
       <c r="D50" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -5184,16 +5184,16 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="G50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0756869904100661)</f>
+        <v>0.0756869904100661</v>
       </c>
       <c r="H50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0756869904100661)</f>
+        <v>0.0756869904100661</v>
       </c>
       <c r="I50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0756869904100661)</f>
+        <v>0.0756869904100661</v>
       </c>
       <c r="J50" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -5208,8 +5208,8 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="M50" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0909796762566006)</f>
+        <v>0.0909796762566006</v>
       </c>
       <c r="N50" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),366.61985757759)</f>
@@ -5358,52 +5358,52 @@
         <v>122</v>
       </c>
       <c r="B52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738143198706873)</f>
+        <v>0.0738143198706873</v>
       </c>
       <c r="C52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
-        <v>0.0875824403367042</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738143198706873)</f>
+        <v>0.0738143198706873</v>
       </c>
       <c r="D52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
-        <v>0.0875824403367042</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826227624746291)</f>
+        <v>0.0826227624746291</v>
       </c>
       <c r="E52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875824403367042)</f>
-        <v>0.0875824403367042</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0945064091827231)</f>
+        <v>0.0945064091827231</v>
       </c>
       <c r="F52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0952134923111048)</f>
+        <v>0.0952134923111048</v>
       </c>
       <c r="G52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0907950767238501)</f>
+        <v>0.0907950767238501</v>
       </c>
       <c r="H52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771791995816322)</f>
+        <v>0.0771791995816322</v>
       </c>
       <c r="I52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782753016610352)</f>
+        <v>0.0782753016610352</v>
       </c>
       <c r="J52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826937172482899)</f>
+        <v>0.0826937172482899</v>
       </c>
       <c r="K52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826937172482899)</f>
+        <v>0.0826937172482899</v>
       </c>
       <c r="L52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819866341199082)</f>
+        <v>0.0819866341199082</v>
       </c>
       <c r="M52" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819169643322097)</f>
-        <v>0.0819169643322097</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864050497071629)</f>
+        <v>0.0864050497071629</v>
       </c>
       <c r="N52" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),300.325058646191)</f>
@@ -5455,52 +5455,52 @@
         <v>123</v>
       </c>
       <c r="B53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738141230528446)</f>
+        <v>0.0738141230528446</v>
       </c>
       <c r="C53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
-        <v>0.0875806052787535</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738141230528446)</f>
+        <v>0.0738141230528446</v>
       </c>
       <c r="D53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
-        <v>0.0875806052787535</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826225891766349)</f>
+        <v>0.0826225891766349</v>
       </c>
       <c r="E53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875806052787535)</f>
-        <v>0.0875806052787535</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0945068249706181)</f>
+        <v>0.0945068249706181</v>
       </c>
       <c r="F53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0952136231283829)</f>
+        <v>0.0952136231283829</v>
       </c>
       <c r="G53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0907952016698743)</f>
+        <v>0.0907952016698743</v>
       </c>
       <c r="H53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.077179442745086)</f>
+        <v>0.077179442745086</v>
       </c>
       <c r="I53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782751122453402)</f>
+        <v>0.0782751122453402</v>
       </c>
       <c r="J53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826935337038488)</f>
+        <v>0.0826935337038488</v>
       </c>
       <c r="K53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826935337038488)</f>
+        <v>0.0826935337038488</v>
       </c>
       <c r="L53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.081986735546084)</f>
+        <v>0.081986735546084</v>
       </c>
       <c r="M53" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819175760181933)</f>
-        <v>0.0819175760181933</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864051570045927)</f>
+        <v>0.0864051570045927</v>
       </c>
       <c r="N53" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),660.71512861809)</f>
@@ -5552,52 +5552,52 @@
         <v>124</v>
       </c>
       <c r="B54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738134657732333)</f>
+        <v>0.0738134657732333</v>
       </c>
       <c r="C54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
-        <v>0.0875791848041027</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738134657732333)</f>
+        <v>0.0738134657732333</v>
       </c>
       <c r="D54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
-        <v>0.0875791848041027</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826224083229981)</f>
+        <v>0.0826224083229981</v>
       </c>
       <c r="E54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875791848041027)</f>
-        <v>0.0875791848041027</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0945072087101559)</f>
+        <v>0.0945072087101559</v>
       </c>
       <c r="F54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0952140122277676)</f>
+        <v>0.0952140122277676</v>
       </c>
       <c r="G54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0907957098996484)</f>
+        <v>0.0907957098996484</v>
       </c>
       <c r="H54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771794819907101)</f>
+        <v>0.0771794819907101</v>
       </c>
       <c r="I54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782752685393762)</f>
+        <v>0.0782752685393762</v>
       </c>
       <c r="J54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826935708674953)</f>
+        <v>0.0826935708674953</v>
       </c>
       <c r="K54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826935708674953)</f>
+        <v>0.0826935708674953</v>
       </c>
       <c r="L54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819867673498837)</f>
+        <v>0.0819867673498837</v>
       </c>
       <c r="M54" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819180495097435)</f>
-        <v>0.0819180495097435</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864050696780028)</f>
+        <v>0.0864050696780028</v>
       </c>
       <c r="N54" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),144.156028161701)</f>
@@ -5608,8 +5608,8 @@
         <v>1</v>
       </c>
       <c r="P54" s="21" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2)</f>
-        <v>2</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3)</f>
+        <v>3</v>
       </c>
       <c r="Q54" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
@@ -5649,52 +5649,52 @@
         <v>125</v>
       </c>
       <c r="B55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738124965393579)</f>
+        <v>0.0738124965393579</v>
       </c>
       <c r="C55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
-        <v>0.0875793661112797</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0738124965393579)</f>
+        <v>0.0738124965393579</v>
       </c>
       <c r="D55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
-        <v>0.0875793661112797</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826224235220467)</f>
+        <v>0.0826224235220467</v>
       </c>
       <c r="E55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0875793661112797)</f>
-        <v>0.0875793661112797</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0945083084729547)</f>
+        <v>0.0945083084729547</v>
       </c>
       <c r="F55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0952145803016424)</f>
+        <v>0.0952145803016424</v>
       </c>
       <c r="G55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0907966823883564)</f>
+        <v>0.0907966823883564</v>
       </c>
       <c r="H55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0771804197218833)</f>
+        <v>0.0771804197218833</v>
       </c>
       <c r="I55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0782751293210692)</f>
+        <v>0.0782751293210692</v>
       </c>
       <c r="J55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826930272343553)</f>
+        <v>0.0826930272343553</v>
       </c>
       <c r="K55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0826930272343553)</f>
+        <v>0.0826930272343553</v>
       </c>
       <c r="L55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819867554056675)</f>
+        <v>0.0819867554056675</v>
       </c>
       <c r="M55" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0819179890740179)</f>
-        <v>0.0819179890740179</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0864046533189536)</f>
+        <v>0.0864046533189536</v>
       </c>
       <c r="N55" s="21" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),96.1040185823099)</f>
@@ -5746,52 +5746,52 @@
         <v>126</v>
       </c>
       <c r="B56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.1015098507676)</f>
-        <v>0.1015098507676</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0948522483704821)</f>
+        <v>0.0948522483704821</v>
       </c>
       <c r="C56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
-        <v>0.0848631221776276</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0815047861926023)</f>
+        <v>0.0815047861926023</v>
       </c>
       <c r="D56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
-        <v>0.0848631221776276</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0764490653204335)</f>
+        <v>0.0764490653204335</v>
       </c>
       <c r="E56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0848631221776276)</f>
-        <v>0.0848631221776276</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0840907184461371)</f>
+        <v>0.0840907184461371</v>
       </c>
       <c r="F56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0847724193282586)</f>
+        <v>0.0847724193282586</v>
       </c>
       <c r="G56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0839123144737292)</f>
+        <v>0.0839123144737292</v>
       </c>
       <c r="H56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0747579341668873)</f>
+        <v>0.0747579341668873</v>
       </c>
       <c r="I56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0754421691956102)</f>
+        <v>0.0754421691956102</v>
       </c>
       <c r="J56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761698137204834)</f>
+        <v>0.0761698137204834</v>
       </c>
       <c r="K56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0761698137204834)</f>
+        <v>0.0761698137204834</v>
       </c>
       <c r="L56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0774844188474166)</f>
-        <v>0.0774844188474166</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0888355750162418)</f>
+        <v>0.0888355750162418</v>
       </c>
       <c r="M56" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.1015098507676)</f>
-        <v>0.1015098507676</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.103043142048651)</f>
+        <v>0.103043142048651</v>
       </c>
       <c r="N56" s="7" t="n">
         <f aca="false">SUM(N39:N55)</f>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="P56" s="7" t="n">
         <f aca="false">SUM(P39:P55)</f>
-        <v>744</v>
+        <v>785</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5903,44 +5903,44 @@
         <v>0.12</v>
       </c>
       <c r="C62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955555555555556)</f>
+        <v>0.0955555555555556</v>
       </c>
       <c r="D62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="E62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="F62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="G62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="H62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="I62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="J62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="K62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0711111111111111)</f>
+        <v>0.0711111111111111</v>
       </c>
       <c r="L62" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.076)</f>
-        <v>0.076</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0955555555555556)</f>
+        <v>0.0955555555555556</v>
       </c>
       <c r="M62" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.12)</f>
@@ -5952,52 +5952,52 @@
         <v>102</v>
       </c>
       <c r="B63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0540540540540541)</f>
+        <v>0.0540540540540541</v>
       </c>
       <c r="C63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0540540540540541)</f>
+        <v>0.0540540540540541</v>
       </c>
       <c r="D63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="E63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="F63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="G63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.108108108108108)</f>
+        <v>0.108108108108108</v>
       </c>
       <c r="H63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="I63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="J63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="K63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="L63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
       <c r="M63" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0810810810810811)</f>
+        <v>0.0810810810810811</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6005,52 +6005,52 @@
         <v>103</v>
       </c>
       <c r="B64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="C64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
-        <v>0.252438087744811</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="D64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
-        <v>0.252438087744811</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.10126582278481)</f>
+        <v>0.10126582278481</v>
       </c>
       <c r="E64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.252438087744811)</f>
-        <v>0.252438087744811</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="F64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="G64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="H64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0886075949367089)</f>
+        <v>0.0886075949367089</v>
       </c>
       <c r="I64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="J64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="K64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="L64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
       <c r="M64" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0269650818628408)</f>
-        <v>0.0269650818628408</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0759493670886076)</f>
+        <v>0.0759493670886076</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6058,52 +6058,52 @@
         <v>104</v>
       </c>
       <c r="B65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="C65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="D65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="E65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="F65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="G65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="H65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0526315789473684)</f>
+        <v>0.0526315789473684</v>
       </c>
       <c r="I65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="J65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="K65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.105263157894737)</f>
+        <v>0.105263157894737</v>
       </c>
       <c r="L65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
       <c r="M65" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0789473684210526)</f>
+        <v>0.0789473684210526</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6164,12 +6164,12 @@
         <v>106</v>
       </c>
       <c r="B67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="C67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="D67" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -6184,16 +6184,16 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="G67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="H67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="I67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="J67" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -6208,8 +6208,8 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="M67" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6217,12 +6217,12 @@
         <v>107</v>
       </c>
       <c r="B68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="C68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="D68" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -6233,20 +6233,20 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="F68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="G68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="H68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="I68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.111111111111111)</f>
+        <v>0.111111111111111</v>
       </c>
       <c r="J68" s="20" t="n">
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
@@ -6257,12 +6257,12 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="L68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
       <c r="M68" s="20" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0833333333333333)</f>
-        <v>0.0833333333333333</v>
+        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0555555555555556)</f>
+        <v>0.0555555555555556</v>
       </c>
     </row>
   </sheetData>
@@ -6318,11 +6318,11 @@
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">MATCH(MAX(Importados!$B$22:$M$22),Importados!$B$22:$M$22,0)</f>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C5" s="24" t="n">
         <f aca="false">MATCH(MAX(Importados!$B$56:$M$56),Importados!$B$56:$M$56,0)</f>
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6331,11 +6331,11 @@
       </c>
       <c r="B6" s="25" t="str">
         <f aca="false">INDEX(Importados!$B$4:$M$4,B5)</f>
-        <v>Ene</v>
+        <v>Dic</v>
       </c>
       <c r="C6" s="25" t="str">
         <f aca="false">INDEX(Importados!$B$38:$M$38,C5)</f>
-        <v>Ene</v>
+        <v>Dic</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6344,11 +6344,11 @@
       </c>
       <c r="B7" s="26" t="n">
         <f aca="false">INDEX(Importados!$B$22:$M$22,B5)</f>
-        <v>0.101848800284409</v>
+        <v>0.102986262617071</v>
       </c>
       <c r="C7" s="26" t="n">
         <f aca="false">INDEX(Importados!$B$56:$M$56,C5)</f>
-        <v>0.1015098507676</v>
+        <v>0.103043142048651</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="F13" s="29" t="n">
         <f aca="false">Importados!$N$5*INDEX(Importados!$B$5:$M$5,$B$5)/$B$8</f>
-        <v>652.692236720059</v>
+        <v>652.618836454199</v>
       </c>
       <c r="G13" s="29" t="n">
         <f aca="false">F13*Importados!$O$5</f>
@@ -6465,11 +6465,11 @@
       </c>
       <c r="H13" s="23" t="n">
         <f aca="false">F13/$C13</f>
-        <v>9.06516995444526</v>
+        <v>9.06415050630832</v>
       </c>
       <c r="I13" s="29" t="n">
         <f aca="false">Importados!$N$39*INDEX(Importados!$B$39:$M$39,$C$5)/$C$8</f>
-        <v>339.292554289086</v>
+        <v>339.254723202532</v>
       </c>
       <c r="J13" s="29" t="n">
         <f aca="false">I13*Importados!$O$39</f>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="K13" s="23" t="n">
         <f aca="false">I13/$C13</f>
-        <v>4.71239658734841</v>
+        <v>4.71187115559072</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>149</v>
@@ -6501,27 +6501,27 @@
       </c>
       <c r="F14" s="29" t="n">
         <f aca="false">Importados!$N$6*INDEX(Importados!$B$6:$M$6,$B$5)/$B$8</f>
-        <v>36.3790897941657</v>
+        <v>37.0808827424103</v>
       </c>
       <c r="G14" s="29" t="n">
         <f aca="false">F14*Importados!$O$6</f>
-        <v>36.3790897941657</v>
+        <v>37.0808827424103</v>
       </c>
       <c r="H14" s="23" t="n">
         <f aca="false">F14/$C14</f>
-        <v>1.21263632647219</v>
+        <v>1.23602942474701</v>
       </c>
       <c r="I14" s="29" t="n">
         <f aca="false">Importados!$N$40*INDEX(Importados!$B$40:$M$40,$C$5)/$C$8</f>
-        <v>18.6772059581256</v>
+        <v>19.2468348066429</v>
       </c>
       <c r="J14" s="29" t="n">
         <f aca="false">I14*Importados!$O$40</f>
-        <v>18.6772059581256</v>
+        <v>19.2468348066429</v>
       </c>
       <c r="K14" s="23" t="n">
         <f aca="false">I14/$C14</f>
-        <v>0.622573531937519</v>
+        <v>0.641561160221431</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>149</v>
@@ -6545,27 +6545,27 @@
       </c>
       <c r="F15" s="29" t="n">
         <f aca="false">Importados!$N$7*INDEX(Importados!$B$7:$M$7,$B$5)/$B$8</f>
-        <v>232.796340138188</v>
+        <v>238.015237592182</v>
       </c>
       <c r="G15" s="29" t="n">
         <f aca="false">F15*Importados!$O$7</f>
-        <v>232.796340138188</v>
+        <v>238.015237592182</v>
       </c>
       <c r="H15" s="23" t="n">
         <f aca="false">F15/$C15</f>
-        <v>9.69984750575784</v>
+        <v>9.9173015663409</v>
       </c>
       <c r="I15" s="29" t="n">
         <f aca="false">Importados!$N$41*INDEX(Importados!$B$41:$M$41,$C$5)/$C$8</f>
-        <v>120.070942594702</v>
+        <v>123.883624610963</v>
       </c>
       <c r="J15" s="29" t="n">
         <f aca="false">I15*Importados!$O$41</f>
-        <v>120.070942594702</v>
+        <v>123.883624610963</v>
       </c>
       <c r="K15" s="23" t="n">
         <f aca="false">I15/$C15</f>
-        <v>5.00295594144594</v>
+        <v>5.16181769212347</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>149</v>
@@ -6589,27 +6589,27 @@
       </c>
       <c r="F16" s="29" t="n">
         <f aca="false">Importados!$N$8*INDEX(Importados!$B$8:$M$8,$B$5)/$B$8</f>
-        <v>12.9711603110206</v>
+        <v>13.8920231904653</v>
       </c>
       <c r="G16" s="29" t="n">
         <f aca="false">F16*Importados!$O$8</f>
-        <v>12.9711603110206</v>
+        <v>13.8920231904653</v>
       </c>
       <c r="H16" s="23" t="n">
         <f aca="false">F16/$C16</f>
-        <v>0.81069751943879</v>
+        <v>0.868251449404081</v>
       </c>
       <c r="I16" s="29" t="n">
         <f aca="false">Importados!$N$42*INDEX(Importados!$B$42:$M$42,$C$5)/$C$8</f>
-        <v>6.65083763296167</v>
+        <v>7.22960704153535</v>
       </c>
       <c r="J16" s="29" t="n">
         <f aca="false">I16*Importados!$O$42</f>
-        <v>6.65083763296167</v>
+        <v>7.22960704153535</v>
       </c>
       <c r="K16" s="23" t="n">
         <f aca="false">I16/$C16</f>
-        <v>0.415677352060105</v>
+        <v>0.451850440095959</v>
       </c>
       <c r="M16" s="5" t="s">
         <v>149</v>
@@ -6633,27 +6633,27 @@
       </c>
       <c r="F17" s="29" t="n">
         <f aca="false">Importados!$N$9*INDEX(Importados!$B$9:$M$9,$B$5)/$B$8</f>
-        <v>18.8029804281169</v>
+        <v>19.6998523581369</v>
       </c>
       <c r="G17" s="29" t="n">
         <f aca="false">F17*Importados!$O$9</f>
-        <v>18.8029804281169</v>
+        <v>19.6998523581369</v>
       </c>
       <c r="H17" s="23" t="n">
         <f aca="false">F17/$C17</f>
-        <v>1.17518627675731</v>
+        <v>1.23124077238356</v>
       </c>
       <c r="I17" s="29" t="n">
         <f aca="false">Importados!$N$43*INDEX(Importados!$B$43:$M$43,$C$5)/$C$8</f>
-        <v>9.6681132372588</v>
+        <v>10.2632365116348</v>
       </c>
       <c r="J17" s="29" t="n">
         <f aca="false">I17*Importados!$O$43</f>
-        <v>9.6681132372588</v>
+        <v>10.2632365116348</v>
       </c>
       <c r="K17" s="23" t="n">
         <f aca="false">I17/$C17</f>
-        <v>0.604257077328675</v>
+        <v>0.641452281977176</v>
       </c>
       <c r="M17" s="5" t="s">
         <v>149</v>
@@ -6809,27 +6809,27 @@
       </c>
       <c r="F21" s="29" t="n">
         <f aca="false">Importados!$N$13*INDEX(Importados!$B$13:$M$13,$B$5)/$B$8</f>
-        <v>8.9191989732046</v>
+        <v>9.58243351095272</v>
       </c>
       <c r="G21" s="29" t="n">
         <f aca="false">F21*Importados!$O$13</f>
-        <v>8.9191989732046</v>
+        <v>9.58243351095272</v>
       </c>
       <c r="H21" s="23" t="n">
         <f aca="false">F21/$C21</f>
-        <v>0.557449935825287</v>
+        <v>0.598902094434545</v>
       </c>
       <c r="I21" s="29" t="n">
         <f aca="false">Importados!$N$47*INDEX(Importados!$B$47:$M$47,$C$5)/$C$8</f>
-        <v>4.55414466197892</v>
+        <v>4.97450118188776</v>
       </c>
       <c r="J21" s="29" t="n">
         <f aca="false">I21*Importados!$O$47</f>
-        <v>4.55414466197892</v>
+        <v>4.97450118188776</v>
       </c>
       <c r="K21" s="23" t="n">
         <f aca="false">I21/$C21</f>
-        <v>0.284634041373682</v>
+        <v>0.310906323867985</v>
       </c>
       <c r="M21" s="5" t="s">
         <v>149</v>
@@ -6853,27 +6853,27 @@
       </c>
       <c r="F22" s="29" t="n">
         <f aca="false">Importados!$N$14*INDEX(Importados!$B$14:$M$14,$B$5)/$B$8</f>
-        <v>49.625920044755</v>
+        <v>51.7478506420602</v>
       </c>
       <c r="G22" s="29" t="n">
         <f aca="false">F22*Importados!$O$14</f>
-        <v>49.625920044755</v>
+        <v>51.7478506420602</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">F22/$C22</f>
-        <v>1.65419733482517</v>
+        <v>1.72492835473534</v>
       </c>
       <c r="I22" s="29" t="n">
         <f aca="false">Importados!$N$48*INDEX(Importados!$B$48:$M$48,$C$5)/$C$8</f>
-        <v>25.4438253440476</v>
+        <v>26.9047032149427</v>
       </c>
       <c r="J22" s="29" t="n">
         <f aca="false">I22*Importados!$O$48</f>
-        <v>25.4438253440476</v>
+        <v>26.9047032149427</v>
       </c>
       <c r="K22" s="23" t="n">
         <f aca="false">I22/$C22</f>
-        <v>0.848127511468254</v>
+        <v>0.896823440498089</v>
       </c>
       <c r="M22" s="5" t="s">
         <v>149</v>
@@ -6897,27 +6897,27 @@
       </c>
       <c r="F23" s="29" t="n">
         <f aca="false">Importados!$N$15*INDEX(Importados!$B$15:$M$15,$B$5)/$B$8</f>
-        <v>17.8150080869683</v>
+        <v>18.4793724972974</v>
       </c>
       <c r="G23" s="29" t="n">
         <f aca="false">F23*Importados!$O$15</f>
-        <v>17.8150080869683</v>
+        <v>18.4793724972974</v>
       </c>
       <c r="H23" s="23" t="n">
         <f aca="false">F23/$C23</f>
-        <v>1.11343800543552</v>
+        <v>1.15496078108109</v>
       </c>
       <c r="I23" s="29" t="n">
         <f aca="false">Importados!$N$49*INDEX(Importados!$B$49:$M$49,$C$5)/$C$8</f>
-        <v>9.23742114169862</v>
+        <v>9.64634335529636</v>
       </c>
       <c r="J23" s="29" t="n">
         <f aca="false">I23*Importados!$O$49</f>
-        <v>9.23742114169862</v>
+        <v>9.64634335529636</v>
       </c>
       <c r="K23" s="23" t="n">
         <f aca="false">I23/$C23</f>
-        <v>0.577338821356164</v>
+        <v>0.602896459706022</v>
       </c>
       <c r="M23" s="5" t="s">
         <v>149</v>
@@ -6941,27 +6941,27 @@
       </c>
       <c r="F24" s="29" t="n">
         <f aca="false">Importados!$N$16*INDEX(Importados!$B$16:$M$16,$B$5)/$B$8</f>
-        <v>2.93881852547358</v>
+        <v>3.14198698162501</v>
       </c>
       <c r="G24" s="29" t="n">
         <f aca="false">F24*Importados!$O$16</f>
-        <v>2.93881852547358</v>
+        <v>3.14198698162501</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">F24/$C24</f>
-        <v>0.122450771894732</v>
+        <v>0.130916124234375</v>
       </c>
       <c r="I24" s="29" t="n">
         <f aca="false">Importados!$N$50*INDEX(Importados!$B$50:$M$50,$C$5)/$C$8</f>
-        <v>1.52758273990662</v>
+        <v>1.66774779758251</v>
       </c>
       <c r="J24" s="29" t="n">
         <f aca="false">I24*Importados!$O$50</f>
-        <v>1.52758273990662</v>
+        <v>1.66774779758251</v>
       </c>
       <c r="K24" s="23" t="n">
         <f aca="false">I24/$C24</f>
-        <v>0.0636492808294427</v>
+        <v>0.0694894915659378</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>149</v>
@@ -7029,27 +7029,27 @@
       </c>
       <c r="F26" s="29" t="n">
         <f aca="false">Importados!$N$18*INDEX(Importados!$B$18:$M$18,$B$5)/$B$8</f>
-        <v>2.37711623910776</v>
+        <v>2.47992147874104</v>
       </c>
       <c r="G26" s="29" t="n">
         <f aca="false">F26*Importados!$O$18</f>
-        <v>2.37711623910776</v>
+        <v>2.47992147874104</v>
       </c>
       <c r="H26" s="23" t="n">
         <f aca="false">F26/$C26</f>
-        <v>1.18855811955388</v>
+        <v>1.23996073937052</v>
       </c>
       <c r="I26" s="29" t="n">
         <f aca="false">Importados!$N$52*INDEX(Importados!$B$52:$M$52,$C$5)/$C$8</f>
-        <v>1.23008585585944</v>
+        <v>1.29748008103154</v>
       </c>
       <c r="J26" s="29" t="n">
         <f aca="false">I26*Importados!$O$52</f>
-        <v>1.23008585585944</v>
+        <v>1.29748008103154</v>
       </c>
       <c r="K26" s="23" t="n">
         <f aca="false">I26/$C26</f>
-        <v>0.61504292792972</v>
+        <v>0.648740040515769</v>
       </c>
       <c r="M26" s="5" t="s">
         <v>152</v>
@@ -7073,27 +7073,27 @@
       </c>
       <c r="F27" s="29" t="n">
         <f aca="false">Importados!$N$19*INDEX(Importados!$B$19:$M$19,$B$5)/$B$8</f>
-        <v>5.22964666029617</v>
+        <v>5.45582081823097</v>
       </c>
       <c r="G27" s="29" t="n">
         <f aca="false">F27*Importados!$O$19</f>
-        <v>5.22964666029617</v>
+        <v>5.45582081823097</v>
       </c>
       <c r="H27" s="23" t="n">
         <f aca="false">F27/$C27</f>
-        <v>2.61482333014809</v>
+        <v>2.72791040911549</v>
       </c>
       <c r="I27" s="29" t="n">
         <f aca="false">Importados!$N$53*INDEX(Importados!$B$53:$M$53,$C$5)/$C$8</f>
-        <v>2.70620908874714</v>
+        <v>2.85445972117779</v>
       </c>
       <c r="J27" s="29" t="n">
         <f aca="false">I27*Importados!$O$53</f>
-        <v>2.70620908874714</v>
+        <v>2.85445972117779</v>
       </c>
       <c r="K27" s="23" t="n">
         <f aca="false">I27/$C27</f>
-        <v>1.35310454437357</v>
+        <v>1.42722986058889</v>
       </c>
       <c r="M27" s="5" t="s">
         <v>152</v>
@@ -7117,27 +7117,27 @@
       </c>
       <c r="F28" s="29" t="n">
         <f aca="false">Importados!$N$20*INDEX(Importados!$B$20:$M$20,$B$5)/$B$8</f>
-        <v>1.14101819180856</v>
+        <v>1.19036240324224</v>
       </c>
       <c r="G28" s="29" t="n">
         <f aca="false">F28*Importados!$O$20</f>
-        <v>1.14101819180856</v>
+        <v>1.19036240324224</v>
       </c>
       <c r="H28" s="23" t="n">
         <f aca="false">F28/$C28</f>
-        <v>0.57050909590428</v>
+        <v>0.595181201621121</v>
       </c>
       <c r="I28" s="29" t="n">
         <f aca="false">Importados!$N$54*INDEX(Importados!$B$54:$M$54,$C$5)/$C$8</f>
-        <v>0.59044903260391</v>
+        <v>0.622790582890795</v>
       </c>
       <c r="J28" s="29" t="n">
         <f aca="false">I28*Importados!$O$54</f>
-        <v>0.59044903260391</v>
+        <v>0.622790582890795</v>
       </c>
       <c r="K28" s="23" t="n">
         <f aca="false">I28/$C28</f>
-        <v>0.295224516301955</v>
+        <v>0.311395291445398</v>
       </c>
       <c r="M28" s="5" t="s">
         <v>152</v>
@@ -7161,27 +7161,27 @@
       </c>
       <c r="F29" s="29" t="n">
         <f aca="false">Importados!$N$21*INDEX(Importados!$B$21:$M$21,$B$5)/$B$8</f>
-        <v>0.760668657682474</v>
+        <v>0.793573755434497</v>
       </c>
       <c r="G29" s="29" t="n">
         <f aca="false">F29*Importados!$O$21</f>
-        <v>0.760668657682474</v>
+        <v>0.793573755434497</v>
       </c>
       <c r="H29" s="23" t="n">
         <f aca="false">F29/$C29</f>
-        <v>0.760668657682474</v>
+        <v>0.793573755434497</v>
       </c>
       <c r="I29" s="29" t="n">
         <f aca="false">Importados!$N$55*INDEX(Importados!$B$55:$M$55,$C$5)/$C$8</f>
-        <v>0.393632397209744</v>
+        <v>0.415191720408138</v>
       </c>
       <c r="J29" s="29" t="n">
         <f aca="false">I29*Importados!$O$55</f>
-        <v>0.393632397209744</v>
+        <v>0.415191720408138</v>
       </c>
       <c r="K29" s="23" t="n">
         <f aca="false">I29/$C29</f>
-        <v>0.393632397209744</v>
+        <v>0.415191720408138</v>
       </c>
       <c r="M29" s="5" t="s">
         <v>152</v>
@@ -7193,27 +7193,27 @@
       </c>
       <c r="F30" s="30" t="n">
         <f aca="false">SUM(F13:F29)</f>
-        <v>1050.21469306323</v>
+        <v>1061.94364471736</v>
       </c>
       <c r="G30" s="30" t="n">
         <f aca="false">SUM(G13:G29)</f>
-        <v>397.522456343171</v>
+        <v>409.324808263162</v>
       </c>
       <c r="H30" s="30" t="n">
         <f aca="false">SUM(H13:H29)</f>
-        <v>31.853123101456</v>
+        <v>32.590797446526</v>
       </c>
       <c r="I30" s="30" t="n">
         <f aca="false">SUM(I13:I29)</f>
-        <v>544.079465849846</v>
+        <v>552.297705704186</v>
       </c>
       <c r="J30" s="30" t="n">
         <f aca="false">SUM(J13:J29)</f>
-        <v>204.786911560761</v>
+        <v>213.042982501654</v>
       </c>
       <c r="K30" s="30" t="n">
         <f aca="false">SUM(K13:K29)</f>
-        <v>16.4682412406882</v>
+        <v>16.97085206833</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7222,11 +7222,11 @@
       </c>
       <c r="F31" s="11" t="n">
         <f aca="false">SUMPRODUCT(F13:F29,$B$13:$B$29)/F30</f>
-        <v>5.61010110978076</v>
+        <v>5.69116685083819</v>
       </c>
       <c r="I31" s="11" t="n">
         <f aca="false">SUMPRODUCT(I13:I29,$B$13:$B$29)/I30</f>
-        <v>5.59545821055644</v>
+        <v>5.69893065809013</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7339,7 +7339,7 @@
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$29:$M$29,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$R$5:$R$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>270.443057759748</v>
+        <v>263.133785928404</v>
       </c>
       <c r="D38" s="22" t="n">
         <f aca="false">Importados!R$23</f>
@@ -7347,15 +7347,15 @@
       </c>
       <c r="E38" s="28" t="n">
         <f aca="false">2*C38/D38</f>
-        <v>36.0590743679664</v>
+        <v>35.0845047904539</v>
       </c>
       <c r="F38" s="28" t="n">
         <f aca="false">E38*(Supuestos!$B$17+Supuestos!$B$18)/60+2*C38*$B38/60</f>
-        <v>34.5566129359678</v>
+        <v>33.6226504241849</v>
       </c>
       <c r="G38" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$63:$M$63,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$R$39:$R$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>139.979837012887</v>
+        <v>136.196598174701</v>
       </c>
       <c r="H38" s="22" t="n">
         <f aca="false">Importados!R$57</f>
@@ -7363,11 +7363,11 @@
       </c>
       <c r="I38" s="28" t="n">
         <f aca="false">2*G38/H38</f>
-        <v>18.663978268385</v>
+        <v>18.1595464232935</v>
       </c>
       <c r="J38" s="28" t="n">
         <f aca="false">I38*(Supuestos!$B$17+Supuestos!$B$18)/60+2*G38*$B38/60</f>
-        <v>17.8863125072023</v>
+        <v>17.4028986556563</v>
       </c>
       <c r="M38" s="5" t="s">
         <v>161</v>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="C39" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$30:$M$30,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$S$5:$S$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>8.34060470826765</v>
+        <v>21.4635570516291</v>
       </c>
       <c r="D39" s="22" t="n">
         <f aca="false">Importados!S$23</f>
@@ -7390,15 +7390,15 @@
       </c>
       <c r="E39" s="28" t="n">
         <f aca="false">2*C39/D39</f>
-        <v>1.39010078471128</v>
+        <v>3.57725950860485</v>
       </c>
       <c r="F39" s="28" t="n">
         <f aca="false">E39*(Supuestos!$B$17+Supuestos!$B$18)/60+2*C39*$B39/60</f>
-        <v>1.22792235982829</v>
+        <v>3.15991256593428</v>
       </c>
       <c r="G39" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$64:$M$64,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$S$39:$S$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>4.72978482937001</v>
+        <v>13.3218273203531</v>
       </c>
       <c r="H39" s="22" t="n">
         <f aca="false">Importados!S$57</f>
@@ -7406,11 +7406,11 @@
       </c>
       <c r="I39" s="28" t="n">
         <f aca="false">2*G39/H39</f>
-        <v>0.788297471561669</v>
+        <v>2.22030455339218</v>
       </c>
       <c r="J39" s="28" t="n">
         <f aca="false">I39*(Supuestos!$B$17+Supuestos!$B$18)/60+2*G39*$B39/60</f>
-        <v>0.696329433212807</v>
+        <v>1.9612690221631</v>
       </c>
       <c r="M39" s="5" t="s">
         <v>161</v>
@@ -7425,7 +7425,7 @@
       </c>
       <c r="C40" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$31:$M$31,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$T$5:$T$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>15.933847507444</v>
+        <v>15.0952239544206</v>
       </c>
       <c r="D40" s="22" t="n">
         <f aca="false">Importados!T$23</f>
@@ -7433,15 +7433,15 @@
       </c>
       <c r="E40" s="28" t="n">
         <f aca="false">2*C40/D40</f>
-        <v>2.89706318317163</v>
+        <v>2.74458617353102</v>
       </c>
       <c r="F40" s="28" t="n">
         <f aca="false">E40*(Supuestos!$B$17+Supuestos!$B$18)/60+2*C40*$B40/60</f>
-        <v>2.48664589888898</v>
+        <v>2.35576979894746</v>
       </c>
       <c r="G40" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$65:$M$65,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$T$39:$T$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>9.32221450894524</v>
+        <v>8.83157164005339</v>
       </c>
       <c r="H40" s="22" t="n">
         <f aca="false">Importados!T$57</f>
@@ -7449,11 +7449,11 @@
       </c>
       <c r="I40" s="28" t="n">
         <f aca="false">2*G40/H40</f>
-        <v>1.6949480925355</v>
+        <v>1.60574029819153</v>
       </c>
       <c r="J40" s="28" t="n">
         <f aca="false">I40*(Supuestos!$B$17+Supuestos!$B$18)/60+2*G40*$B40/60</f>
-        <v>1.45483044609297</v>
+        <v>1.37826042261439</v>
       </c>
       <c r="M40" s="5" t="s">
         <v>161</v>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="C42" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$33:$M$33,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$V$5:$V$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>23.6691084679195</v>
+        <v>31.5588112905594</v>
       </c>
       <c r="D42" s="22" t="n">
         <f aca="false">Importados!V$23</f>
@@ -7519,15 +7519,15 @@
       </c>
       <c r="E42" s="28" t="n">
         <f aca="false">2*C42/D42</f>
-        <v>0.776036343210476</v>
+        <v>1.03471512428063</v>
       </c>
       <c r="F42" s="28" t="n">
         <f aca="false">E42*(Supuestos!$B$17+Supuestos!$B$18)/60+2*C42*$B42/60</f>
-        <v>1.63614329026875</v>
+        <v>2.181524387025</v>
       </c>
       <c r="G42" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$67:$M$67,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$V$39:$V$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>13.8301471124783</v>
+        <v>18.4401961499711</v>
       </c>
       <c r="H42" s="22" t="n">
         <f aca="false">Importados!V$57</f>
@@ -7535,11 +7535,11 @@
       </c>
       <c r="I42" s="28" t="n">
         <f aca="false">2*G42/H42</f>
-        <v>0.453447446310765</v>
+        <v>0.60459659508102</v>
       </c>
       <c r="J42" s="28" t="n">
         <f aca="false">I42*(Supuestos!$B$17+Supuestos!$B$18)/60+2*G42*$B42/60</f>
-        <v>0.956018365971863</v>
+        <v>1.27469115462915</v>
       </c>
       <c r="M42" s="5" t="s">
         <v>161</v>
@@ -7554,7 +7554,7 @@
       </c>
       <c r="C43" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$34:$M$34,$B$5)*SUMPRODUCT(Importados!$N$5:$N$21,Importados!$W$5:$W$21/Importados!$X$5:$X$21)/$B$8</f>
-        <v>3.40742438250904</v>
+        <v>2.27161625500603</v>
       </c>
       <c r="D43" s="22" t="n">
         <f aca="false">Importados!W$23</f>
@@ -7562,15 +7562,15 @@
       </c>
       <c r="E43" s="28" t="n">
         <f aca="false">2*C43/D43</f>
-        <v>1.13580812750301</v>
+        <v>0.757205418335343</v>
       </c>
       <c r="F43" s="28" t="n">
         <f aca="false">E43*(Supuestos!$B$17+Supuestos!$B$18)/60+2*C43*$B43/60</f>
-        <v>0.776135553793726</v>
+        <v>0.517423702529151</v>
       </c>
       <c r="G43" s="29" t="n">
         <f aca="false">INDEX(Importados!$B$68:$M$68,$C$5)*SUMPRODUCT(Importados!$N$39:$N$55,Importados!$W$39:$W$55/Importados!$X$39:$X$55)/$C$8</f>
-        <v>2.12990990117672</v>
+        <v>1.41993993411782</v>
       </c>
       <c r="H43" s="22" t="n">
         <f aca="false">Importados!W$57</f>
@@ -7578,11 +7578,11 @@
       </c>
       <c r="I43" s="28" t="n">
         <f aca="false">2*G43/H43</f>
-        <v>0.709969967058907</v>
+        <v>0.473313311372605</v>
       </c>
       <c r="J43" s="28" t="n">
         <f aca="false">I43*(Supuestos!$B$17+Supuestos!$B$18)/60+2*G43*$B43/60</f>
-        <v>0.48514614415692</v>
+        <v>0.32343076277128</v>
       </c>
       <c r="M43" s="5" t="s">
         <v>161</v>
@@ -7594,27 +7594,27 @@
       </c>
       <c r="C44" s="30" t="n">
         <f aca="false">SUM(C37:C43)</f>
-        <v>1050.21469306323</v>
+        <v>1061.94364471736</v>
       </c>
       <c r="E44" s="30" t="n">
         <f aca="false">SUM(E37:E43)</f>
-        <v>202.933635977327</v>
+        <v>203.873824185969</v>
       </c>
       <c r="F44" s="30" t="n">
         <f aca="false">SUM(F37:F43)</f>
-        <v>148.344763881951</v>
+        <v>149.498584721824</v>
       </c>
       <c r="G44" s="30" t="n">
         <f aca="false">SUM(G37:G43)</f>
-        <v>544.079465849848</v>
+        <v>552.297705704187</v>
       </c>
       <c r="I44" s="30" t="n">
         <f aca="false">SUM(I37:I43)</f>
-        <v>104.932589629389</v>
+        <v>105.685449564868</v>
       </c>
       <c r="J44" s="30" t="n">
         <f aca="false">SUM(J37:J43)</f>
-        <v>76.6725012481408</v>
+        <v>77.5344143693381</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7634,11 +7634,11 @@
       </c>
       <c r="B49" s="29" t="n">
         <f aca="false">F30</f>
-        <v>1050.21469306323</v>
+        <v>1061.94364471736</v>
       </c>
       <c r="C49" s="29" t="n">
         <f aca="false">I30</f>
-        <v>544.079465849846</v>
+        <v>552.297705704186</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7647,11 +7647,11 @@
       </c>
       <c r="B50" s="29" t="n">
         <f aca="false">G30</f>
-        <v>397.522456343171</v>
+        <v>409.324808263162</v>
       </c>
       <c r="C50" s="29" t="n">
         <f aca="false">J30</f>
-        <v>204.786911560761</v>
+        <v>213.042982501654</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7660,11 +7660,11 @@
       </c>
       <c r="B51" s="29" t="n">
         <f aca="false">B49+B50</f>
-        <v>1447.7371494064</v>
+        <v>1471.26845298052</v>
       </c>
       <c r="C51" s="29" t="n">
         <f aca="false">C49+C50</f>
-        <v>748.866377410607</v>
+        <v>765.34068820584</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7673,11 +7673,11 @@
       </c>
       <c r="B52" s="28" t="n">
         <f aca="false">F31</f>
-        <v>5.61010110978076</v>
+        <v>5.69116685083819</v>
       </c>
       <c r="C52" s="28" t="n">
         <f aca="false">I31</f>
-        <v>5.59545821055644</v>
+        <v>5.69893065809013</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7686,11 +7686,11 @@
       </c>
       <c r="B53" s="31" t="n">
         <f aca="false">H30/F30</f>
-        <v>0.0303301061314881</v>
+        <v>0.0306897617483272</v>
       </c>
       <c r="C53" s="31" t="n">
         <f aca="false">K30/I30</f>
-        <v>0.0302680808123589</v>
+        <v>0.0307277250893012</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7699,11 +7699,11 @@
       </c>
       <c r="B54" s="21" t="n">
         <f aca="false">Supuestos!$B$6/(B53*Supuestos!$B$24)</f>
-        <v>172.020212581163</v>
+        <v>170.004294824225</v>
       </c>
       <c r="C54" s="21" t="n">
         <f aca="false">Supuestos!$B$6/(C53*Supuestos!$B$24)</f>
-        <v>172.372716218515</v>
+        <v>169.794258741413</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7712,11 +7712,11 @@
       </c>
       <c r="B55" s="21" t="n">
         <f aca="false">Supuestos!$B$11/B52</f>
-        <v>249.549869530732</v>
+        <v>245.995247845142</v>
       </c>
       <c r="C55" s="21" t="n">
         <f aca="false">Supuestos!$B$11/C52</f>
-        <v>250.202923034748</v>
+        <v>245.66012187086</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7725,11 +7725,11 @@
       </c>
       <c r="B56" s="21" t="n">
         <f aca="false">MIN(B54,B55)</f>
-        <v>172.020212581163</v>
+        <v>170.004294824225</v>
       </c>
       <c r="C56" s="21" t="n">
         <f aca="false">MIN(C54,C55)</f>
-        <v>172.372716218515</v>
+        <v>169.794258741413</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7738,11 +7738,11 @@
       </c>
       <c r="B57" s="23" t="n">
         <f aca="false">B51/B56</f>
-        <v>8.41608743346555</v>
+        <v>8.65430167221207</v>
       </c>
       <c r="C57" s="23" t="n">
         <f aca="false">C51/C56</f>
-        <v>4.34446003891518</v>
+        <v>4.50745916781208</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7751,11 +7751,11 @@
       </c>
       <c r="B58" s="28" t="n">
         <f aca="false">E44</f>
-        <v>202.933635977327</v>
+        <v>203.873824185969</v>
       </c>
       <c r="C58" s="28" t="n">
         <f aca="false">I44</f>
-        <v>104.932589629389</v>
+        <v>105.685449564868</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7764,11 +7764,11 @@
       </c>
       <c r="B59" s="28" t="n">
         <f aca="false">F44</f>
-        <v>148.344763881951</v>
+        <v>149.498584721824</v>
       </c>
       <c r="C59" s="28" t="n">
         <f aca="false">J44</f>
-        <v>76.6725012481408</v>
+        <v>77.5344143693381</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7777,11 +7777,11 @@
       </c>
       <c r="B60" s="23" t="n">
         <f aca="false">B59/($B$9-Supuestos!$B$16)</f>
-        <v>24.7241273136584</v>
+        <v>24.9164307869707</v>
       </c>
       <c r="C60" s="23" t="n">
         <f aca="false">C59/($C$9-Supuestos!$B$16)</f>
-        <v>12.7787502080235</v>
+        <v>12.9224023948897</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7803,11 +7803,11 @@
       </c>
       <c r="B62" s="28" t="n">
         <f aca="false">B61*Supuestos!$B$16+B59</f>
-        <v>185.844763881951</v>
+        <v>186.998584721824</v>
       </c>
       <c r="C62" s="28" t="n">
         <f aca="false">C61*Supuestos!$B$16+C59</f>
-        <v>96.1725012481408</v>
+        <v>97.0344143693381</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7829,11 +7829,11 @@
       </c>
       <c r="B64" s="32" t="n">
         <f aca="false">B62/(B63*$B$9*Supuestos!$B$15)</f>
-        <v>0.884975066104527</v>
+        <v>0.890469451056304</v>
       </c>
       <c r="C64" s="32" t="n">
         <f aca="false">C62/(C63*$C$9*Supuestos!$B$15)</f>
-        <v>0.801437510401173</v>
+        <v>0.808620119744484</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7842,11 +7842,11 @@
       </c>
       <c r="B65" s="21" t="n">
         <f aca="false">B51*B52/B61</f>
-        <v>324.878071542227</v>
+        <v>334.92936993147</v>
       </c>
       <c r="C65" s="21" t="n">
         <f aca="false">C51*C52/C61</f>
-        <v>322.326963083987</v>
+        <v>335.509500915389</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7924,31 +7924,31 @@
       </c>
       <c r="B70" s="21" t="n">
         <f aca="false">F30*Supuestos!$B$22</f>
-        <v>525.107346531615</v>
+        <v>530.97182235868</v>
       </c>
       <c r="C70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*H13:H29)*Supuestos!$B$22*Supuestos!$B$24</f>
-        <v>14.8076127992378</v>
+        <v>15.1040870788577</v>
       </c>
       <c r="D70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*H13:H29)*Supuestos!$B$22</f>
-        <v>3.05037650791249</v>
+        <v>3.16140995903894</v>
       </c>
       <c r="E70" s="22" t="n">
         <f aca="false">ROUNDUP(C70,0)+ROUNDUP(D70,0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F70" s="21" t="n">
         <f aca="false">I30*Supuestos!$B$22</f>
-        <v>272.039732924923</v>
+        <v>276.148852852093</v>
       </c>
       <c r="G70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*K13:K29)*Supuestos!$B$22*Supuestos!$B$24</f>
-        <v>7.65268321403531</v>
+        <v>7.857991736822</v>
       </c>
       <c r="H70" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*K13:K29)*Supuestos!$B$22</f>
-        <v>1.57961347770469</v>
+        <v>1.6523897412763</v>
       </c>
       <c r="I70" s="22" t="n">
         <f aca="false">ROUNDUP(G70,0)+ROUNDUP(H70,0)</f>
@@ -7964,31 +7964,31 @@
       </c>
       <c r="B71" s="21" t="n">
         <f aca="false">F30*Supuestos!$B$23</f>
-        <v>525.107346531615</v>
+        <v>530.97182235868</v>
       </c>
       <c r="C71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*H13:H29)*Supuestos!$B$23*Supuestos!$B$24</f>
-        <v>14.8076127992378</v>
+        <v>15.1040870788577</v>
       </c>
       <c r="D71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*H13:H29)*Supuestos!$B$23</f>
-        <v>3.05037650791249</v>
+        <v>3.16140995903894</v>
       </c>
       <c r="E71" s="22" t="n">
         <f aca="false">ROUNDUP(C71,0)+ROUNDUP(D71,0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F71" s="21" t="n">
         <f aca="false">I30*Supuestos!$B$23</f>
-        <v>272.039732924923</v>
+        <v>276.148852852093</v>
       </c>
       <c r="G71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*K13:K29)*Supuestos!$B$23*Supuestos!$B$24</f>
-        <v>7.65268321403531</v>
+        <v>7.857991736822</v>
       </c>
       <c r="H71" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*K13:K29)*Supuestos!$B$23</f>
-        <v>1.57961347770469</v>
+        <v>1.6523897412763</v>
       </c>
       <c r="I71" s="22" t="n">
         <f aca="false">ROUNDUP(G71,0)+ROUNDUP(H71,0)</f>
@@ -8004,15 +8004,15 @@
       </c>
       <c r="B72" s="21" t="n">
         <f aca="false">G30</f>
-        <v>397.522456343171</v>
+        <v>409.324808263162</v>
       </c>
       <c r="C72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*G13:G29/$C$13:$C$29)</f>
-        <v>16.6872001311857</v>
+        <v>17.2038270221398</v>
       </c>
       <c r="D72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*G13:G29/$C$13:$C$29)</f>
-        <v>6.10075301582498</v>
+        <v>6.32281991807788</v>
       </c>
       <c r="E72" s="22" t="n">
         <f aca="false">ROUNDUP(C72/Supuestos!$B$26,0)+ROUNDUP(D72,0)</f>
@@ -8020,15 +8020,15 @@
       </c>
       <c r="F72" s="21" t="n">
         <f aca="false">J30</f>
-        <v>204.786911560761</v>
+        <v>213.042982501654</v>
       </c>
       <c r="G72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=0)*J13:J29/$C$13:$C$29)</f>
-        <v>8.59661769793039</v>
+        <v>8.95420143018668</v>
       </c>
       <c r="H72" s="28" t="n">
         <f aca="false">SUMPRODUCT(($E$13:$E$29=1)*J13:J29/$C$13:$C$29)</f>
-        <v>3.15922695540939</v>
+        <v>3.3047794825526</v>
       </c>
       <c r="I72" s="22" t="n">
         <f aca="false">ROUNDUP(G72/Supuestos!$B$26,0)+ROUNDUP(H72,0)</f>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="E74" s="9" t="n">
         <f aca="false">SUM(E70:E73)</f>
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I74" s="9" t="n">
         <f aca="false">SUM(I70:I73)</f>
@@ -8091,7 +8091,7 @@
       </c>
       <c r="E75" s="11" t="n">
         <f aca="false">E74*Supuestos!$B$28</f>
-        <v>127.2</v>
+        <v>132</v>
       </c>
       <c r="I75" s="11" t="n">
         <f aca="false">I74*Supuestos!$B$28</f>
@@ -8104,11 +8104,11 @@
       </c>
       <c r="E76" s="7" t="n">
         <f aca="false">Importados!$P$22</f>
-        <v>1384</v>
+        <v>1498</v>
       </c>
       <c r="I76" s="7" t="n">
         <f aca="false">Importados!$P$56</f>
-        <v>744</v>
+        <v>785</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8117,11 +8117,11 @@
       </c>
       <c r="E77" s="9" t="n">
         <f aca="false">ROUNDUP(SUM(C70:C72),0)+B63*Supuestos!$B$6+E73*Supuestos!$B$27</f>
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I77" s="9" t="n">
         <f aca="false">ROUNDUP(SUM(G70:G72),0)+C63*Supuestos!$B$6+I73*Supuestos!$B$27</f>
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>